<commit_message>
update pipline output short
</commit_message>
<xml_diff>
--- a/output/testcases_e2e_short_vb.xlsx
+++ b/output/testcases_e2e_short_vb.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>1. kết nối tổng đài viên giúp mình</t>
+          <t>1. cho anh gặp tồng đài viên</t>
         </is>
       </c>
       <c r="H5" s="3" t="n"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>1. cho anh gặp tồng đài viên</t>
+          <t>1. chuyển máy cho tổng đài viên giúp anh</t>
         </is>
       </c>
       <c r="H6" s="3" t="n"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>1. chết rồi</t>
+          <t>1. mới ốm mất rồi em ạ</t>
         </is>
       </c>
       <c r="H7" s="3" t="n"/>
@@ -810,7 +810,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>1. ừ mất rôi em thông cảm</t>
+          <t>1. đột quỵ chết rồi em ạ</t>
         </is>
       </c>
       <c r="H8" s="3" t="n"/>
@@ -854,7 +854,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>1. cho gặp nhân viên tư vấn đi em</t>
+          <t>1. chuyển máy cho tổng đài viên giúp anh</t>
         </is>
       </c>
       <c r="H9" s="3" t="n"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>1. ốm chết rồi</t>
+          <t>1. chết rồi</t>
         </is>
       </c>
       <c r="H10" s="3" t="n"/>
@@ -939,8 +939,8 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>1. lúc khác rồi nói
-2. đi học rồi</t>
+          <t>1. lát rồi gọi lại
+2. không nói chuyện được</t>
         </is>
       </c>
       <c r="H11" s="3" t="n"/>
@@ -988,9 +988,9 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>1. ai đấy nhỉ
-2. alo ai đang gọi vậy
-3. alo ai đang gọi vậy</t>
+          <t>1. ai đấy alo ạ
+2. ai đấy
+3. ai đấy alo ạ</t>
         </is>
       </c>
       <c r="H12" s="3" t="n"/>
@@ -1038,8 +1038,8 @@
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>1. ai đấy alo ạ
-2. ai đấy nhỉ
-3. alo ai đang gọi vậy</t>
+2. ai đấy
+3. ai đấy alo ạ</t>
         </is>
       </c>
       <c r="H13" s="3" t="n"/>
@@ -1087,9 +1087,9 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>1. ai đấy alo ạ
-2. ai đấy
-3. alo ai đấy ạ</t>
+          <t>1. ai đấy
+2. alo ai đấy ạ
+3. ai đấy</t>
         </is>
       </c>
       <c r="H14" s="3" t="n"/>
@@ -1172,8 +1172,8 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1. cút mẹ mày đi
-2. sao mày ngu thế</t>
+          <t>1. mày có cút không
+2. con thần kinh</t>
         </is>
       </c>
       <c r="H16" s="3" t="n"/>
@@ -1219,8 +1219,8 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>1. nói lại giúm mình với nãy không nghe thấy
-2. không nghe thấy gì hết trơn á</t>
+          <t>1. alo alo nghe không có rõ
+2. nghe không rõ nói lại đi em</t>
         </is>
       </c>
       <c r="H17" s="3" t="n"/>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>1. nói lại giúm mình với nãy không nghe thấy
+          <t>1. tín hiệu kém quá không nghe thấy gì
 2. nghe không rõ nói lại đi em</t>
         </is>
       </c>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>1. nói lại được không em
+          <t>1. chẳng nghe thấy gì
 2. chẳng nghe thấy gì</t>
         </is>
       </c>
@@ -1378,8 +1378,8 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. mới ung thư mất rồi</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. mất rồi em</t>
         </is>
       </c>
       <c r="H21" s="3" t="n"/>
@@ -1425,7 +1425,7 @@
       <c r="G22" s="3" t="inlineStr">
         <is>
           <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. chết rồi</t>
+2. mới ung thư mất rồi</t>
         </is>
       </c>
       <c r="H22" s="3" t="n"/>
@@ -1472,7 +1472,7 @@
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>1. bố cháu đang nghe
-2. mất rồi em</t>
+2. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
         </is>
       </c>
       <c r="H23" s="3" t="n"/>
@@ -1515,9 +1515,9 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. đang có việc
-3. lúc khác rồi nói</t>
+          <t>1. anh nghe hộ thôi
+2. anh đang đi trên đường
+3. bận rồi</t>
         </is>
       </c>
       <c r="H24" s="3" t="n"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. bố cháu đang nghe
 2. _silence_
 3. _silence_</t>
         </is>
@@ -1610,9 +1610,9 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. nghe không rõ nói lại đi em
-3. alo alo nghe không có rõ</t>
+          <t>1. nó đi vắng rồi chưa về
+2. chẳng nghe thấy gì
+3. nghe không rõ nói lại đi em</t>
         </is>
       </c>
       <c r="H26" s="3" t="n"/>
@@ -1659,9 +1659,9 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. nói bé quá nói lại đi em
-3. không nghe thấy gì hết trơn á</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. nghe không rõ nói lại đi em
+3. chẳng nghe thấy gì</t>
         </is>
       </c>
       <c r="H27" s="3" t="n"/>
@@ -1709,9 +1709,9 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. alo alo nghe không có rõ
-3. chẳng nghe thấy gì</t>
+          <t>1. nó đi chơi rồi
+2. nghe không rõ nói lại đi em
+3. nói lại được không em</t>
         </is>
       </c>
       <c r="H28" s="3" t="n"/>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. anh nghe hộ thôi
 2. không phải số này
 3. không phải số này</t>
         </is>
@@ -1808,9 +1808,9 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. không phải rồi
-3. gọi sai người rồi</t>
+          <t>1. đang nghe hộ không biết đâu
+2. nhầm số rồi
+3. nhầm rồi em ơi</t>
         </is>
       </c>
       <c r="H30" s="3" t="n"/>
@@ -1858,9 +1858,9 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. không phải rồi
-3. nhầm số rồi</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. không phải số này
+3. có phải anh đâu</t>
         </is>
       </c>
       <c r="H31" s="3" t="n"/>
@@ -1922,8 +1922,8 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
 3. ủa đã trả rồi mà em</t>
         </is>
       </c>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
+          <t>1. nó ra ngoài rồi
 2. có có quen có việc gì không
 3. anh muốn mở lại thẻ ấy em</t>
         </is>
@@ -2023,8 +2023,8 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. có có quen có việc gì không
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ ừ người quen
 3. được miễn lãi mấy hôm em</t>
         </is>
       </c>
@@ -2073,9 +2073,9 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ ừ người quen
-3. anh còn nợ bao tiền đã trả được nhiều chưa</t>
+          <t>1. anh nghe hộ thôi
+2. có quen sao em
+3. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H36" s="3" t="n"/>
@@ -2123,9 +2123,9 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. anh biết bạn ấy có gì không
-3. tải app home như nào</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
+3. thanh toán qua app như nào</t>
         </is>
       </c>
       <c r="H37" s="3" t="n"/>
@@ -2173,9 +2173,9 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. tôi là anh nó
 2. ừ ừ người quen
-3. chuyển máy cho tư vấn viên</t>
+3. cho mình gặp tư vấn viên</t>
         </is>
       </c>
       <c r="H38" s="3" t="n"/>
@@ -2222,8 +2222,8 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. anh biết bạn ấy có gì không
+          <t>1. tôi là anh nó
+2. ừ ừ người quen
 3. thẻ anh bị khoá em mở ra giúp anh với</t>
         </is>
       </c>
@@ -2271,9 +2271,9 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. có có quen có việc gì không
-3. miễn lãi nhiều ngày không em</t>
+          <t>1. bố cháu đang nghe
+2. có quen sao em
+3. miễn lãi mấy hôm</t>
         </is>
       </c>
       <c r="H40" s="3" t="n"/>
@@ -2320,9 +2320,9 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có có quen có việc gì không
-3. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ ừ người quen
+3. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H41" s="3" t="n"/>
@@ -2370,8 +2370,8 @@
       <c r="G42" s="3" t="inlineStr">
         <is>
           <t>1. nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. thanh toán qua app như nào</t>
+2. có quen sao em
+3. cách tải app như nào</t>
         </is>
       </c>
       <c r="H42" s="3" t="n"/>
@@ -2418,9 +2418,9 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. nó đi vắng rồi chưa về
 2. có có quen có việc gì không
-3. chuyển máy cho tư vấn viên</t>
+3. cho mình gặp tư vấn viên</t>
         </is>
       </c>
       <c r="H43" s="3" t="n"/>
@@ -2468,9 +2468,9 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ừ ừ người quen
-3. chết rồi</t>
+          <t>1. nó đi chơi rồi
+2. có có quen có việc gì không
+3. tại nạn chết rồi em</t>
         </is>
       </c>
       <c r="H44" s="3" t="n"/>
@@ -2517,9 +2517,9 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ người quen
-3. đột quỵ chết rồi em ạ</t>
+          <t>1. tôi là anh nó
+2. có quen sao em
+3. mất rồi em</t>
         </is>
       </c>
       <c r="H45" s="3" t="n"/>
@@ -2562,9 +2562,9 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. đang khó khăn tôi không trả</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
+3. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H46" s="3" t="n"/>
@@ -2612,9 +2612,9 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ừ tôi có biết
-3. mở lại thẻ giúp anh</t>
+          <t>1. nó đi chơi rồi
+2. có quen sao em
+3. thẻ anh bị khoá em mở ra giúp anh với</t>
         </is>
       </c>
       <c r="H47" s="3" t="n"/>
@@ -2663,9 +2663,9 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. ừ tôi có biết
-3. miễn lãi mấy hôm</t>
+3. được miễn lãi mấy hôm em</t>
         </is>
       </c>
       <c r="H48" s="3" t="n"/>
@@ -2713,8 +2713,8 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
+          <t>1. nó đi vắng rồi chưa về
+2. có quen sao em
 3. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
@@ -2763,8 +2763,8 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có quen sao em
+          <t>1. anh nghe hộ thôi
+2. anh biết bạn ấy có gì không
 3. cách tải app như nào</t>
         </is>
       </c>
@@ -2813,9 +2813,9 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ người quen
-3. chuyển máy cho tư vấn viên</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. có quen sao em
+3. cho mình gặp tư vấn viên</t>
         </is>
       </c>
       <c r="H51" s="3" t="n"/>
@@ -2863,8 +2863,8 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. có quen sao em
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ ừ người quen
 3. ốm chết rồi</t>
         </is>
       </c>
@@ -2917,11 +2917,11 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. anh biết bạn ấy có gì không
-3. quẹt gì
-4. mua gì
-5. mua gì</t>
+3. giao dịch cái gì
+4. quẹt gì
+5. giao dịch cái gì</t>
         </is>
       </c>
       <c r="H53" s="3" t="n"/>
@@ -2972,11 +2972,11 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. có quen sao em
+          <t>1. tôi là anh nó
+2. có có quen có việc gì không
 3. giao dịch cái gì
-4. quẹt gì
-5. quẹt gì</t>
+4. tiền gì
+5. mua gì</t>
         </is>
       </c>
       <c r="H54" s="3" t="n"/>
@@ -3028,11 +3028,11 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. có có quen có việc gì không
-3. mua gì
-4. quẹt gì
-5. quẹt gì</t>
+          <t>1. anh nghe hộ thôi
+2. anh biết bạn ấy có gì không
+3. quẹt gì
+4. tiền gì
+5. tiền gì</t>
         </is>
       </c>
       <c r="H55" s="3" t="n"/>
@@ -3084,11 +3084,11 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
+          <t>1. đang nghe hộ không biết đâu
 2. ừ ừ người quen
-3. số hợp đồng là gì em
+3. hợp đồng mã số là gì
 4. số hợp đồng của anh là bao nhiêu
-5. số hợp đồng của anh là bao nhiêu</t>
+5. hợp đồng mã số là gì</t>
         </is>
       </c>
       <c r="H56" s="3" t="n"/>
@@ -3140,10 +3140,10 @@
       <c r="G57" s="3" t="inlineStr">
         <is>
           <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ ừ người quen
-3. số hợp đồng là gì em
-4. số hợp đồng của anh là bao nhiêu
-5. hợp đồng mã số là gì</t>
+2. ừ tôi có biết
+3. hợp đồng mã số là gì
+4. hợp đồng mã số là gì
+5. số hợp đồng của anh là bao nhiêu</t>
         </is>
       </c>
       <c r="H57" s="3" t="n"/>
@@ -3195,9 +3195,9 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ tôi có biết
-3. hợp đồng mã số là gì
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ ừ người quen
+3. số hợp đồng là gì em
 4. số hợp đồng của anh là bao nhiêu
 5. số hợp đồng là gì em</t>
         </is>
@@ -3244,10 +3244,10 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. có quen sao em
-3. anh đang bận
-4. bận rồi</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
+3. đi học rồi
+4. chưa tiện để nói chuyện</t>
         </is>
       </c>
       <c r="H59" s="3" t="n"/>
@@ -3299,11 +3299,11 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. có có quen có việc gì không
-3. có trả góp được không
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
+3. anh muốn chuyển sang trả góp được không
 4. giờ trả góp có được không em
-5. có trả góp được không</t>
+5. giờ trả góp có được không em</t>
         </is>
       </c>
       <c r="H60" s="3" t="n"/>
@@ -3354,9 +3354,9 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. ừ tôi có biết
-3. anh muốn chuyển sang trả góp được không
+3. giờ trả góp có được không em
 4. giờ trả góp có được không em
 5. anh muốn chuyển sang trả góp được không</t>
         </is>
@@ -3410,11 +3410,11 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ người quen
-3. có trả góp được không
+          <t>1. nó ra ngoài rồi
+2. có quen sao em
+3. anh muốn chuyển sang trả góp được không
 4. anh muốn chuyển sang trả góp được không
-5. anh muốn chuyển sang trả góp được không</t>
+5. giờ trả góp có được không em</t>
         </is>
       </c>
       <c r="H62" s="3" t="n"/>
@@ -3466,10 +3466,10 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ người quen
-3. hạn mức thẻ là bao nhiêu em
-4. hạn mức thẻ có cao không máy chục thế em
+          <t>1. bố cháu đang nghe
+2. có quen sao em
+3. hạn mức thẻ có cao không máy chục thế em
+4. thẻ có những hạn mức nào em
 5. thẻ có những hạn mức nào em</t>
         </is>
       </c>
@@ -3521,11 +3521,11 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ ừ người quen
-3. hạn mức thẻ là bao nhiêu em
-4. hạn mức thẻ là bao nhiêu em
-5. thẻ có những hạn mức nào em</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. có quen sao em
+3. hạn mức thẻ có cao không máy chục thế em
+4. hạn mức thẻ có cao không máy chục thế em
+5. hạn mức thẻ có cao không máy chục thế em</t>
         </is>
       </c>
       <c r="H64" s="3" t="n"/>
@@ -3577,10 +3577,10 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. nó ra ngoài rồi
 2. anh biết bạn ấy có gì không
-3. hạn mức thẻ là bao nhiêu em
-4. hạn mức thẻ là bao nhiêu em
+3. thẻ có những hạn mức nào em
+4. hạn mức thẻ có cao không máy chục thế em
 5. hạn mức thẻ có cao không máy chục thế em</t>
         </is>
       </c>
@@ -3633,8 +3633,8 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. anh biết bạn ấy có gì không
+          <t>1. nó đi chơi rồi
+2. ừ tôi có biết
 3. anh không dùng thẻ huỷ cho anh nhé
 4. anh không dùng thẻ huỷ cho anh nhé
 5. anh không có dùng huỷ thẻ giúp anh</t>
@@ -3688,11 +3688,11 @@
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. bố cháu đang nghe
 2. có quen sao em
-3. anh không có dùng huỷ thẻ giúp anh
-4. anh không có dùng huỷ thẻ giúp anh
-5. huỷ thẻ giúp anh</t>
+3. anh không dùng thẻ huỷ cho anh nhé
+4. anh không dùng thẻ huỷ cho anh nhé
+5. anh không dùng thẻ huỷ cho anh nhé</t>
         </is>
       </c>
       <c r="H67" s="3" t="n"/>
@@ -3744,11 +3744,11 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ tôi có biết
-3. anh không có dùng huỷ thẻ giúp anh
-4. anh không có dùng huỷ thẻ giúp anh
-5. huỷ thẻ giúp anh</t>
+          <t>1. bố cháu đang nghe
+2. có quen sao em
+3. huỷ thẻ giúp anh
+4. huỷ thẻ giúp anh
+5. anh không dùng thẻ huỷ cho anh nhé</t>
         </is>
       </c>
       <c r="H68" s="3" t="n"/>
@@ -3800,11 +3800,11 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ tôi có biết
-3. thanh toán bằng mo mo được không
-4. thanh toán online được không em
-5. anh trả qua zalo pay có được không</t>
+          <t>1. anh nghe hộ thôi
+2. có quen sao em
+3. anh trả qua zalo pay có được không
+4. chuyển khoản được không em
+5. thanh toán online được không em</t>
         </is>
       </c>
       <c r="H69" s="3" t="n"/>
@@ -3855,10 +3855,10 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. anh biết bạn ấy có gì không
-3. thanh toán bằng mo mo được không
-4. thanh toán online được không em
+          <t>1. nó đi vắng rồi chưa về
+2. có có quen có việc gì không
+3. chuyển khoản được không em
+4. chuyển khoản được không em
 5. thanh toán online được không em</t>
         </is>
       </c>
@@ -3911,11 +3911,11 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
+          <t>1. nó đi chơi rồi
 2. ừ ừ người quen
-3. thanh toán online được không em
-4. thanh toán bằng mo mo được không
-5. thanh toán bằng mo mo được không</t>
+3. anh trả qua zalo pay có được không
+4. thanh toán online được không em
+5. thanh toán online được không em</t>
         </is>
       </c>
       <c r="H71" s="3" t="n"/>
@@ -3967,11 +3967,11 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. có có quen có việc gì không
-3. tổng lãi chị phải trả là bao nhiêu
-4. lãi vay tính như nào vậy em
-5. lãi suất này đã bao gồm hết chi phí chưa em</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ ừ người quen
+3. lãi tính theo dư nợ gốc hay dư nợ giảm dần vậy
+4. vay nhiều lãi có cao hơn không em
+5. lãi suất bên mình như thế nào thế em</t>
         </is>
       </c>
       <c r="H72" s="3" t="n"/>
@@ -4022,11 +4022,11 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
+          <t>1. đang nghe hộ không biết đâu
 2. có có quen có việc gì không
-3. vay nhiều lãi có cao hơn không em
-4. vay nhiều lãi có cao hơn không em
-5. lãi suất bên mình như thế nào thế em</t>
+3. lãi xuất có cố định không em
+4. tổng lãi chị phải trả là bao nhiêu
+5. lãi xuất có cố định không em</t>
         </is>
       </c>
       <c r="H73" s="3" t="n"/>
@@ -4078,11 +4078,11 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có quen sao em
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
 3. tổng lãi chị phải trả là bao nhiêu
-4. lãi vay tính như nào vậy em
-5. tính lãi như nào vậy em</t>
+4. lãi suất bên mình như thế nào thế em
+5. lãi xuất có cố định không em</t>
         </is>
       </c>
       <c r="H74" s="3" t="n"/>
@@ -4134,10 +4134,10 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. anh biết bạn ấy có gì không
+          <t>1. nó đi vắng rồi chưa về
+2. có quen sao em
 3. lãi suất chuyển đổi trả góp có cao không
-4. lãi suất suất chuyển đổi trả góp như nào thế
+4. lãi suất chuyển đổi trả góp có cao không
 5. lãi suất suất chuyển đổi trả góp như nào thế</t>
         </is>
       </c>
@@ -4189,8 +4189,8 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ ừ người quen
+          <t>1. bố cháu đang nghe
+2. anh biết bạn ấy có gì không
 3. lãi suất suất chuyển đổi trả góp như nào thế
 4. lãi suất suất chuyển đổi trả góp như nào thế
 5. lãi suất chuyển đổi trả góp có cao không</t>
@@ -4245,11 +4245,11 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
+          <t>1. nó đi vắng rồi chưa về
 2. ừ tôi có biết
-3. lãi suất suất chuyển đổi trả góp như nào thế
+3. lãi suất chuyển đổi trả góp nhiêu em
 4. lãi suất suất chuyển đổi trả góp như nào thế
-5. lãi suất chuyển đổi trả góp nhiêu em</t>
+5. lãi suất suất chuyển đổi trả góp như nào thế</t>
         </is>
       </c>
       <c r="H77" s="3" t="n"/>
@@ -4301,10 +4301,10 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. có quen sao em
-3. anh làm mất thẻ rồi em ạ
-4. anh mất thẻ rồi
+          <t>1. nó ra ngoài rồi
+2. ừ ừ người quen
+3. mất thẻ thì giờ như nào
+4. anh làm rơi mất thẻ lâu rồi
 5. anh làm mất thẻ rồi em ạ</t>
         </is>
       </c>
@@ -4356,11 +4356,11 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
-3. anh mất thẻ rồi
-4. anh làm mất thẻ rồi em ạ
-5. anh làm rơi mất thẻ lâu rồi</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ừ tôi có biết
+3. anh làm mất thẻ rồi em ạ
+4. anh mất thẻ rồi
+5. anh làm mất thẻ rồi em ạ</t>
         </is>
       </c>
       <c r="H79" s="3" t="n"/>
@@ -4412,11 +4412,11 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. có có quen có việc gì không
 3. mất thẻ thì giờ như nào
-4. anh làm rơi mất thẻ lâu rồi
-5. anh mất thẻ rồi</t>
+4. mất thẻ thì giờ như nào
+5. anh làm rơi mất thẻ lâu rồi</t>
         </is>
       </c>
       <c r="H80" s="3" t="n"/>
@@ -4468,10 +4468,10 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
-3. ngày mấy chốt sao kê em
-4. chốt sao kê ngày nào
+          <t>1. nó đi vắng rồi chưa về
+2. có có quen có việc gì không
+3. chốt sao kê ngày nào
+4. ngày chốt sao kê là ngày mấy
 5. ngày mấy chốt sao kê em</t>
         </is>
       </c>
@@ -4523,11 +4523,11 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. có có quen có việc gì không
-3. chốt sao kê ngày nào
-4. hôm nào chốt sao kê em nhỉ
-5. ngày mấy chốt sao kê em</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ừ tôi có biết
+3. ngày chốt sao kê là ngày mấy
+4. ngày chốt sao kê là ngày mấy
+5. hôm nào chốt sao kê em nhỉ</t>
         </is>
       </c>
       <c r="H82" s="3" t="n"/>
@@ -4579,11 +4579,11 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. có quen sao em
+          <t>1. nó đi vắng rồi chưa về
+2. ừ tôi có biết
 3. ngày chốt sao kê là ngày mấy
-4. ngày chốt sao kê là ngày mấy
-5. ngày mấy chốt sao kê em</t>
+4. hôm nào chốt sao kê em nhỉ
+5. hôm nào chốt sao kê em nhỉ</t>
         </is>
       </c>
       <c r="H83" s="3" t="n"/>
@@ -4635,11 +4635,11 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
-3. hạn đóng tiền là hôm nào
-4. hạn trả là ngày mấy
-5. hôm nào đến hạn thanh toán em</t>
+          <t>1. nó đi vắng rồi chưa về
+2. có có quen có việc gì không
+3. hạn chót thanh toán là hôm nào
+4. hạn chót thanh toán là hôm nào
+5. hạn chót thanh toán là hôm nào</t>
         </is>
       </c>
       <c r="H84" s="3" t="n"/>
@@ -4690,11 +4690,11 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. có có quen có việc gì không
-3. hạn chót để trà là ngày mấy
+          <t>1. nó đi vắng rồi chưa về
+2. ừ tôi có biết
+3. hạn trả là ngày mấy
 4. hạn chót thanh toán là hôm nào
-5. hôm nào đến hạn thanh toán em</t>
+5. hạn trả là ngày mấy</t>
         </is>
       </c>
       <c r="H85" s="3" t="n"/>
@@ -4746,10 +4746,10 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. anh biết bạn ấy có gì không
-3. hạn đóng tiền là hôm nào
-4. hạn đóng tiền là hôm nào
+          <t>1. nó ra ngoài rồi
+2. có có quen có việc gì không
+3. hạn chót thanh toán là hôm nào
+4. hôm nào đến hạn thanh toán em
 5. hạn chót để trà là ngày mấy</t>
         </is>
       </c>
@@ -4802,11 +4802,11 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có quen sao em
-3. ý là phí thường bên em lấy như nào
-4. phí thường niên cao không em
-5. ý là phí thường bên em lấy như nào</t>
+          <t>1. nó đi vắng rồi chưa về
+2. có có quen có việc gì không
+3. phí thường niên cao không em
+4. ý là phí thường bên em lấy như nào
+5. phí thường niên là bao nhiêu</t>
         </is>
       </c>
       <c r="H87" s="3" t="n"/>
@@ -4857,11 +4857,11 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
+          <t>1. nó đi chơi rồi
 2. anh biết bạn ấy có gì không
-3. phí thường niên cao không em
-4. phí thường niên cao không em
-5. phí thường niên là bao nhiêu</t>
+3. phí thường niên là bao nhiêu
+4. ý là phí thường bên em lấy như nào
+5. phí thường niên cao không em</t>
         </is>
       </c>
       <c r="H88" s="3" t="n"/>
@@ -4914,7 +4914,7 @@
       <c r="G89" s="3" t="inlineStr">
         <is>
           <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. có quen sao em
+2. có có quen có việc gì không
 3. ý là phí thường bên em lấy như nào
 4. ý là phí thường bên em lấy như nào
 5. phí thường niên là bao nhiêu</t>
@@ -4969,11 +4969,11 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
+          <t>1. nó đi chơi rồi
 2. anh biết bạn ấy có gì không
-3. rút tiền kiểu gì em nhỉ
+3. giờ anh muốn rút tiền mặt âý
 4. rút tiền kiểu gì em nhỉ
-5. anh muốn rút tiền mặt ấy</t>
+5. rút tiền mặt như nào em</t>
         </is>
       </c>
       <c r="H90" s="3" t="n"/>
@@ -5024,11 +5024,11 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có quen sao em
-3. giờ anh muốn rút tiền mặt âý
-4. anh muốn rút tiền mặt ấy
-5. giờ anh muốn rút tiền mặt âý</t>
+          <t>1. bố cháu đang nghe
+2. ừ ừ người quen
+3. rút tiền kiểu gì em nhỉ
+4. rút tiền mặt như nào em
+5. anh muốn rút tiền mặt ấy</t>
         </is>
       </c>
       <c r="H91" s="3" t="n"/>
@@ -5080,11 +5080,11 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ tôi có biết
-3. giờ anh muốn rút tiền mặt âý
-4. rút tiền mặt như nào em
-5. rút tiền kiểu gì em nhỉ</t>
+          <t>1. nó ra ngoài rồi
+2. có quen sao em
+3. anh muốn rút tiền mặt ấy
+4. anh muốn rút tiền mặt ấy
+5. giờ anh muốn rút tiền mặt âý</t>
         </is>
       </c>
       <c r="H92" s="3" t="n"/>
@@ -5136,11 +5136,11 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ tôi có biết
+          <t>1. anh nghe hộ thôi
+2. có quen sao em
 3. sản phẩm gì em
-4. sản phẩm gì em
-5. sản phẩm gì em</t>
+4. sản phẩm vay gì đây
+5. em gọi giới thiệu sản phẩm gì</t>
         </is>
       </c>
       <c r="H93" s="3" t="n"/>
@@ -5192,10 +5192,10 @@
       <c r="G94" s="3" t="inlineStr">
         <is>
           <t>1. nó ra ngoài rồi
-2. ừ tôi có biết
+2. có quen sao em
 3. sản phẩm gì em
-4. em gọi giới thiệu sản phẩm gì
-5. sản phẩm vay gì đây</t>
+4. sản phẩm gì em
+5. em gọi giới thiệu sản phẩm gì</t>
         </is>
       </c>
       <c r="H94" s="3" t="n"/>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
 2. có quen sao em
 3. sản phẩm gì em
 4. sản phẩm vay gì đây
@@ -5303,11 +5303,11 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. anh biết bạn ấy có gì không
-3. khoản này trễ mấy hôm rồi em nhỉ
-4. anh trả trễ mấy hôm rồi
-5. anh trả trễ mấy hôm rồi</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. có quen sao em
+3. khoản này trễ mấy hôm rồi
+4. khoản này trễ mấy hôm rồi em nhỉ
+5. khoản này trễ mấy hôm rồi</t>
         </is>
       </c>
       <c r="H96" s="3" t="n"/>
@@ -5358,8 +5358,8 @@
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có có quen có việc gì không
+          <t>1. tôi là anh nó
+2. anh biết bạn ấy có gì không
 3. anh trả trễ mấy hôm rồi
 4. khoản này trễ mấy hôm rồi em nhỉ
 5. nợ trễ lâu chưa em</t>
@@ -5414,11 +5414,11 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. khoản này trễ mấy hôm rồi
-4. anh trả trễ mấy hôm rồi
-5. anh trả trễ mấy hôm rồi</t>
+          <t>1. nó đi chơi rồi
+2. ừ ừ người quen
+3. khoản này trễ mấy hôm rồi em nhỉ
+4. khoản này trễ mấy hôm rồi em nhỉ
+5. nợ trễ lâu chưa em</t>
         </is>
       </c>
       <c r="H98" s="3" t="n"/>
@@ -5470,11 +5470,11 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. có quen sao em
-3. tra lại giao dịch hộ anh với
-4. ừ kiểm tra lại giao dịch giúp anh với
-5. em tra lại giao dịch giúp anh nhé</t>
+          <t>1. anh nghe hộ thôi
+2. ừ tôi có biết
+3. em tra lại giao dịch giúp anh nhé
+4. em tra lại giao dịch giúp anh nhé
+5. ừ kiểm tra lại giao dịch giúp anh với</t>
         </is>
       </c>
       <c r="H99" s="3" t="n"/>
@@ -5525,11 +5525,11 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
-3. ừ kiểm tra lại giao dịch giúp anh với
-4. tra lại giao dịch hộ anh với
-5. ừ kiểm tra lại giao dịch giúp anh với</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
+3. tra lại giao dịch hộ anh với
+4. em tra lại giao dịch giúp anh nhé
+5. tra lại giao dịch hộ anh với</t>
         </is>
       </c>
       <c r="H100" s="3" t="n"/>
@@ -5581,11 +5581,11 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
-3. tra lại giao dịch hộ anh với
+          <t>1. anh nghe hộ thôi
+2. ừ tôi có biết
+3. em tra lại giao dịch giúp anh nhé
 4. em tra lại giao dịch giúp anh nhé
-5. tra lại giao dịch hộ anh với</t>
+5. ừ kiểm tra lại giao dịch giúp anh với</t>
         </is>
       </c>
       <c r="H101" s="3" t="n"/>
@@ -5641,11 +5641,11 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. có có quen có việc gì không
-3. tiền đợt trước khác đợt này lại khác hả em
-4. tiền đợt trước khác đợt này lại khác hả em
-5. số tiền kỳ này lại khác đợt trước à em</t>
+          <t>1. bố cháu đang nghe
+2. anh biết bạn ấy có gì không
+3. sao tiền kỳ này lại khác kỳ trước hả em
+4. sao tiền kỳ này lại khác kỳ trước hả em
+5. tiền đợt trước khác đợt này lại khác hả em</t>
         </is>
       </c>
       <c r="H102" s="3" t="n"/>
@@ -5700,11 +5700,11 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. có có quen có việc gì không
-3. sao tiền kỳ này lại khác kỳ trước hả em
+          <t>1. nó đi vắng rồi chưa về
+2. anh biết bạn ấy có gì không
+3. tiền đợt trước khác đợt này lại khác hả em
 4. tiền đợt trước khác đợt này lại khác hả em
-5. tiền đợt trước khác đợt này lại khác hả em</t>
+5. sao tiền kỳ này lại khác kỳ trước hả em</t>
         </is>
       </c>
       <c r="H103" s="3" t="n"/>
@@ -5760,11 +5760,11 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ tôi có biết
-3. tiền đợt trước khác đợt này lại khác hả em
+          <t>1. nó ra ngoài rồi
+2. có có quen có việc gì không
+3. số tiền kỳ này lại khác đợt trước à em
 4. số tiền kỳ này lại khác đợt trước à em
-5. số tiền kỳ này lại khác đợt trước à em</t>
+5. tiền đợt trước khác đợt này lại khác hả em</t>
         </is>
       </c>
       <c r="H104" s="3" t="n"/>
@@ -5816,8 +5816,8 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. anh biết bạn ấy có gì không
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
 3. em bên nào nhở
 4. em bên nào gọi đến vậy em
 5. em bên nào gọi đến vậy em</t>
@@ -5871,8 +5871,8 @@
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. có quen sao em
+          <t>1. bố cháu đang nghe
+2. ừ tôi có biết
 3. em bên nào nhở
 4. em bên ngân hàng nào đấy
 5. em bên ngân hàng nào đấy</t>
@@ -5927,11 +5927,11 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. em bên ngân hàng nào đấy
+          <t>1. bố cháu đang nghe
+2. ừ ừ người quen
+3. em bên nào nhở
 4. em bên nào gọi đến vậy em
-5. em bên nào gọi đến vậy em</t>
+5. em bên nào nhở</t>
         </is>
       </c>
       <c r="H107" s="3" t="n"/>
@@ -5983,11 +5983,11 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. có có quen có việc gì không
-3. lãi phạt cao không
+          <t>1. nó đi chơi rồi
+2. anh biết bạn ấy có gì không
+3. lãi phạt như nào em
 4. lãi phạt cao không
-5. có lãi phạt hả em bao nhiêu</t>
+5. lãi phạt cao không</t>
         </is>
       </c>
       <c r="H108" s="3" t="n"/>
@@ -6038,11 +6038,11 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. anh biết bạn ấy có gì không
+          <t>1. nó đi vắng rồi chưa về
+2. có quen sao em
 3. lãi phạt cao không
 4. có lãi phạt hả em bao nhiêu
-5. lãi phạt cao không</t>
+5. có lãi phạt hả em bao nhiêu</t>
         </is>
       </c>
       <c r="H109" s="3" t="n"/>
@@ -6094,10 +6094,10 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. anh biết bạn ấy có gì không
-3. lãi phạt cao không
-4. lãi phạt như nào em
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có quen sao em
+3. có lãi phạt hả em bao nhiêu
+4. lãi phạt cao không
 5. có lãi phạt hả em bao nhiêu</t>
         </is>
       </c>
@@ -6150,10 +6150,10 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. hôm nay ngày mấy em
-4. hôm nay là ngày bao nhiêu
+          <t>1. nó ra ngoài rồi
+2. có có quen có việc gì không
+3. hôm nay là ngày bao nhiêu
+4. hôm nay ngày mấy em
 5. hôm nay là ngày bao nhiêu</t>
         </is>
       </c>
@@ -6205,11 +6205,11 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. có quen sao em
-3. hôm nay là ngày bao nhiêu
-4. hôm nay ngày mấy em
-5. hôm nay là ngày bao nhiêu</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ tôi có biết
+3. hôm nay ngày mấy em
+4. hôm nay là ngày bao nhiêu
+5. hôm nay ngày mấy em</t>
         </is>
       </c>
       <c r="H112" s="3" t="n"/>
@@ -6261,11 +6261,11 @@
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ ừ người quen
+          <t>1. anh nghe hộ thôi
+2. có có quen có việc gì không
 3. hôm nay là ngày bao nhiêu
 4. hôm nay ngày mấy em
-5. hôm nay ngày mấy em</t>
+5. hôm nay là ngày bao nhiêu</t>
         </is>
       </c>
       <c r="H113" s="3" t="n"/>
@@ -6317,11 +6317,11 @@
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ tôi có biết
+          <t>1. nó đi chơi rồi
+2. có quen sao em
 3. phí dùng thẻ như nào em em
-4. phí dùng thẻ như nào em em
-5. phí dùng thẻ như nào em em</t>
+4. dùng thẻ thì phí bao nhiêu em
+5. dùng thẻ thì phí bao nhiêu em</t>
         </is>
       </c>
       <c r="H114" s="3" t="n"/>
@@ -6373,10 +6373,10 @@
       <c r="G115" s="3" t="inlineStr">
         <is>
           <t>1. tôi là anh nó
-2. ừ ừ người quen
-3. dùng thẻ thì phí bao nhiêu em
-4. dùng thẻ thì phí bao nhiêu em
-5. dùng thẻ thì phí bao nhiêu em</t>
+2. ừ tôi có biết
+3. phí dùng thẻ như nào
+4. phí dùng thẻ như nào
+5. phí dùng thẻ như nào</t>
         </is>
       </c>
       <c r="H115" s="3" t="n"/>
@@ -6428,10 +6428,10 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ tôi có biết
+          <t>1. bố cháu đang nghe
+2. anh biết bạn ấy có gì không
 3. phí dùng thẻ như nào
-4. phí dùng thẻ như nào em em
+4. phí dùng thẻ như nào
 5. phí dùng thẻ như nào</t>
         </is>
       </c>
@@ -6485,10 +6485,10 @@
       <c r="G117" s="3" t="inlineStr">
         <is>
           <t>1. nó đi vắng rồi chưa về
-2. anh biết bạn ấy có gì không
+2. ừ tôi có biết
 3. tối thiểu cần thanh toán nhiêu em
 4. cần trả it nhất bao nhiêu em
-5. giờ tối thiểu phải thanh toán bao tiền</t>
+5. cần trả it nhất bao nhiêu em</t>
         </is>
       </c>
       <c r="H117" s="3" t="n"/>
@@ -6539,11 +6539,11 @@
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. có có quen có việc gì không
-3. tối thiểu cần thanh toán nhiêu em
-4. tối thiểu cần thanh toán nhiêu em
-5. cân thanh toán tối thiểu bao nhiêu tiền em</t>
+          <t>1. nó đi chơi rồi
+2. có quen sao em
+3. giờ tối thiểu phải thanh toán bao tiền
+4. cân thanh toán tối thiểu bao nhiêu tiền em
+5. tối thiểu cần thanh toán nhiêu em</t>
         </is>
       </c>
       <c r="H118" s="3" t="n"/>
@@ -6595,9 +6595,9 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. cân thanh toán tối thiểu bao nhiêu tiền em
+          <t>1. tôi là anh nó
+2. có có quen có việc gì không
+3. tối thiểu cần thanh toán nhiêu em
 4. giờ tối thiểu phải thanh toán bao tiền
 5. tối thiểu cần thanh toán nhiêu em</t>
         </is>
@@ -6651,11 +6651,11 @@
       </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. có quen sao em
+          <t>1. bố cháu đang nghe
+2. anh biết bạn ấy có gì không
 3. dư nợ cuối kì nhu nào em
-4. dư nợ cuối kì nhu nào em
-5. dư nợ nhiêu em</t>
+4. dư nợ nhiêu em
+5. dư nợ cuối kì nhu nào em</t>
         </is>
       </c>
       <c r="H120" s="3" t="n"/>
@@ -6706,10 +6706,10 @@
       </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. đang nghe hộ không biết đâu
 2. ừ ừ người quen
-3. dư nợ cuối kì nhu nào em
-4. dư nợ cuối kì nhu nào em
+3. dư nợ nhiêu em
+4. tông dư nợ là bao nhiêu em
 5. tông dư nợ là bao nhiêu em</t>
         </is>
       </c>
@@ -6763,9 +6763,9 @@
       <c r="G122" s="3" t="inlineStr">
         <is>
           <t>1. bố cháu đang nghe
-2. có quen sao em
-3. dư nợ cuối kì nhu nào em
-4. dư nợ nhiêu em
+2. ừ tôi có biết
+3. tông dư nợ là bao nhiêu em
+4. tông dư nợ là bao nhiêu em
 5. tông dư nợ là bao nhiêu em</t>
         </is>
       </c>
@@ -6816,8 +6816,8 @@
       </c>
       <c r="G123" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ ừ người quen
+          <t>1. tôi là anh nó
+2. anh biết bạn ấy có gì không
 3. _silence_
 4. _silence_</t>
         </is>
@@ -6868,8 +6868,8 @@
       </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ người quen
+          <t>1. nó ra ngoài rồi
+2. có có quen có việc gì không
 3. _silence_
 4. _silence_</t>
         </is>
@@ -6921,8 +6921,8 @@
       </c>
       <c r="G125" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ người quen
+          <t>1. nó ra ngoài rồi
+2. anh biết bạn ấy có gì không
 3. _silence_
 4. _silence_</t>
         </is>
@@ -6976,10 +6976,10 @@
       </c>
       <c r="G126" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ừ tôi có biết
+          <t>1. anh nghe hộ thôi
+2. anh biết bạn ấy có gì không
 3. bớt nợ cho anh được không dạo này khó khắn quá em
-4. kẹt quá có bớt nợ cho anh được không
+4. bớt nợ cho anh được không dạo này khó khắn quá em
 5. bớt nợ cho anh được không dạo này khó khắn quá em</t>
         </is>
       </c>
@@ -7031,11 +7031,11 @@
       </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ tôi có biết
+          <t>1. nó đi vắng rồi chưa về
+2. ừ ừ người quen
 3. giảm nợ cho anh được không
-4. kẹt quá có bớt nợ cho anh được không
-5. bớt nợ cho anh được không dạo này khó khắn quá em</t>
+4. giảm nợ cho anh được không
+5. giảm nợ cho anh được không</t>
         </is>
       </c>
       <c r="H127" s="3" t="n"/>
@@ -7087,10 +7087,10 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. có quen sao em
+          <t>1. anh nghe hộ thôi
+2. anh biết bạn ấy có gì không
 3. bớt nợ cho anh được không dạo này khó khắn quá em
-4. giảm nợ cho anh được không
+4. kẹt quá có bớt nợ cho anh được không
 5. bớt nợ cho anh được không dạo này khó khắn quá em</t>
         </is>
       </c>
@@ -7141,10 +7141,10 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ người quen
+          <t>1. nó đi chơi rồi
+2. có quen sao em
 3. mấy hôm nữa thanh toán nhé
-4. mấy hôm nữa thanh toán nhé</t>
+4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
       <c r="H129" s="3" t="n"/>
@@ -7194,10 +7194,10 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. có có quen có việc gì không
+          <t>1. nó ra ngoài rồi
+2. có quen sao em
 3. ừ tháng sau trả nhé
-4. anh trả cho bên em sau không bùng đâu yên tâm</t>
+4. ừ tháng sau trả nhé</t>
         </is>
       </c>
       <c r="H130" s="3" t="n"/>
@@ -7247,9 +7247,9 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ tôi có biết
-3. anh trả cho bên em sau không bùng đâu yên tâm
+          <t>1. nó ra ngoài rồi
+2. có có quen có việc gì không
+3. ừ tháng sau trả nhé
 4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
@@ -7302,11 +7302,11 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ ừ người quen
-3. em gửi cho anh tin nhắn nhé
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
+3. gửi tin nhắn giúp anh nhé
 4. gửi lại tin qua zalo hay gì cho anh nhé
-5. gửi lại tin qua zalo hay gì cho anh nhé</t>
+5. gửi tin nhắn giúp anh nhé</t>
         </is>
       </c>
       <c r="H132" s="3" t="n"/>
@@ -7357,11 +7357,11 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
+          <t>1. nó ra ngoài rồi
 2. anh biết bạn ấy có gì không
-3. gửi lại tin qua zalo hay gì cho anh nhé
+3. gửi tin nhắn giúp anh nhé
 4. gửi tin nhắn giúp anh nhé
-5. gửi tin nhắn giúp anh nhé</t>
+5. em gửi cho anh tin nhắn nhé</t>
         </is>
       </c>
       <c r="H133" s="3" t="n"/>
@@ -7413,11 +7413,11 @@
       </c>
       <c r="G134" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ người quen
+          <t>1. nó đi chơi rồi
+2. có có quen có việc gì không
 3. gửi lại tin qua zalo hay gì cho anh nhé
-4. em gửi cho anh tin nhắn nhé
-5. gửi lại tin qua zalo hay gì cho anh nhé</t>
+4. gửi lại tin qua zalo hay gì cho anh nhé
+5. gửi tin nhắn giúp anh nhé</t>
         </is>
       </c>
       <c r="H134" s="3" t="n"/>
@@ -7467,10 +7467,10 @@
       </c>
       <c r="G135" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ừ ừ người quen
-3. nói lại giúm mình với nãy không nghe thấy
-4. nói lại giúm mình với nãy không nghe thấy</t>
+          <t>1. nó ra ngoài rồi
+2. anh biết bạn ấy có gì không
+3. nói bé quá nói lại đi em
+4. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H135" s="3" t="n"/>
@@ -7519,8 +7519,8 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ người quen
+          <t>1. nó đi chơi rồi
+2. có có quen có việc gì không
 3. tín hiệu kém quá không nghe thấy gì
 4. nói bé quá nói lại đi em</t>
         </is>
@@ -7573,8 +7573,8 @@
       <c r="G137" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. có có quen có việc gì không
-3. không nghe thấy gì hết trơn á
+2. anh biết bạn ấy có gì không
+3. alo alo nghe không có rõ
 4. alo alo nghe không có rõ</t>
         </is>
       </c>
@@ -7627,11 +7627,11 @@
       </c>
       <c r="G138" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ừ ừ người quen
-3. mày có cút không
-4. con thần kinh
-5. óc lợn à</t>
+          <t>1. anh nghe hộ thôi
+2. có quen sao em
+3. biến bà mày đi
+4. cút mẹ mày đi
+5. mày bị ngu à</t>
         </is>
       </c>
       <c r="H138" s="3" t="n"/>
@@ -7683,10 +7683,10 @@
       <c r="G139" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. anh biết bạn ấy có gì không
+2. ừ tôi có biết
 3. mày bị ngu à
-4. sao mày ngu thế
-5. sao mày ngu thế</t>
+4. mày bị ngu à
+5. mày điếc à</t>
         </is>
       </c>
       <c r="H139" s="3" t="n"/>
@@ -7738,11 +7738,11 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. nó đi chơi rồi
 2. ừ tôi có biết
 3. mày bị ngu à
-4. óc lợn à
-5. mày có cút không</t>
+4. con điên kia
+5. sao mày ngu thế</t>
         </is>
       </c>
       <c r="H140" s="3" t="n"/>
@@ -7794,10 +7794,10 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
 2. anh biết bạn ấy có gì không
-3. anh điện bên em bằng số nào
-4. hotline bên em là số nào
+3. hotline bên em là số nào
+4. số hotline là gì em nhỉ
 5. hotline bên em là số nào</t>
         </is>
       </c>
@@ -7850,10 +7850,10 @@
       <c r="G142" s="3" t="inlineStr">
         <is>
           <t>1. anh nghe hộ thôi
-2. có có quen có việc gì không
+2. ừ ừ người quen
 3. số hotline là gì em nhỉ
-4. số hotline là gì em nhỉ
-5. số hotline là gì em nhỉ</t>
+4. hotline bên em là số nào
+5. hotline bên em là số nào</t>
         </is>
       </c>
       <c r="H142" s="3" t="n"/>
@@ -7905,11 +7905,11 @@
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. có có quen có việc gì không
+          <t>1. nó đi chơi rồi
+2. có quen sao em
 3. hotline bên em là số nào
-4. anh điện bên em bằng số nào
-5. anh điện bên em bằng số nào</t>
+4. hotline bên em là số nào
+5. số hotline là gì em nhỉ</t>
         </is>
       </c>
       <c r="H143" s="3" t="n"/>
@@ -7961,11 +7961,11 @@
       </c>
       <c r="G144" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. anh nghe hộ thôi
 2. anh biết bạn ấy có gì không
-3. gọi nhiều mắc phiền
-4. sao cứ gọi hoài vậy đừng gọi nữa
-5. suốt ngày gọi</t>
+3. suốt ngày gọi
+4. gọi hoài
+5. gọi hoài</t>
         </is>
       </c>
       <c r="H144" s="3" t="n"/>
@@ -8016,11 +8016,11 @@
       </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ người quen
-3. gọi nhiều mắc phiền
-4. sao cứ gọi hoài vậy đừng gọi nữa
-5. gọi hoài</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ tôi có biết
+3. sao cứ gọi hoài vậy đừng gọi nữa
+4. suốt ngày gọi
+5. suốt ngày gọi</t>
         </is>
       </c>
       <c r="H145" s="3" t="n"/>
@@ -8073,10 +8073,10 @@
       <c r="G146" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. ừ tôi có biết
+2. ừ ừ người quen
 3. gọi hoài
-4. gọi hoài
-5. suốt ngày gọi</t>
+4. gọi nhiều mắc phiền
+5. gọi hoài</t>
         </is>
       </c>
       <c r="H146" s="3" t="n"/>
@@ -8140,10 +8140,10 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ tôi có biết
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. thanh toán rồi mà em ơi</t>
+          <t>1. nó đi vắng rồi chưa về
+2. có có quen có việc gì không
+3. trả trước một phần có được không em
+4. thanh toán xong hết rồi nhá</t>
         </is>
       </c>
       <c r="H148" s="3" t="n"/>
@@ -8193,10 +8193,10 @@
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. anh biết bạn ấy có gì không
-3. anh thanh toán một ít trước nhé
-4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. có quen sao em
+3. trả trước một phần có được không em
+4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H149" s="3" t="n"/>
@@ -8245,10 +8245,10 @@
       </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. có quen sao em
-3. trả trước một phần có được không em
-4. anh trả được nhiêu còn nợ nhiêu em</t>
+          <t>1. bố cháu đang nghe
+2. có có quen có việc gì không
+3. thanh toán một phần trước nhé em
+4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H150" s="3" t="n"/>
@@ -8293,10 +8293,10 @@
       </c>
       <c r="G151" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ người quen
-3. trả trước một phần có được không em
-4. không trả không có tiền</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ tôi có biết
+3. thanh toán một phần trước nhé em
+4. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H151" s="3" t="n"/>
@@ -8346,10 +8346,10 @@
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. nó đi vắng rồi chưa về
 2. ừ tôi có biết
-3. anh thanh toán một ít trước nhé
-4. mất rồi em</t>
+3. anh thanh toán cho bên em trước một phần có được không
+4. đột quỵ chết rồi em ạ</t>
         </is>
       </c>
       <c r="H152" s="3" t="n"/>
@@ -8398,10 +8398,10 @@
       </c>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ tôi có biết
-3. trả trước một phần có được không em
-4. ốm chết rồi</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. đột quỵ chết rồi em ạ</t>
         </is>
       </c>
       <c r="H153" s="3" t="n"/>
@@ -8451,9 +8451,9 @@
       </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. bố cháu đang nghe
 2. ừ ừ người quen
-3. trả trước một phần có được không em
+3. thanh toán một phần trước nhé em
 4. anh trả được nhiêu còn nợ nhiêu em</t>
         </is>
       </c>
@@ -8504,10 +8504,10 @@
       </c>
       <c r="G155" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. anh biết bạn ấy có gì không
-3. giờ trả được một ít trước thôi em
-4. mới ung thư mất rồi</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. có có quen có việc gì không
+3. anh thanh toán cho bên em trước một phần có được không
+4. tại nạn chết rồi em</t>
         </is>
       </c>
       <c r="H155" s="3" t="n"/>
@@ -8556,10 +8556,10 @@
       </c>
       <c r="G156" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. anh biết bạn ấy có gì không
-3. thanh toán một phần trước nhé em
-4. được để anh trả tiền</t>
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. ừ anh thanh toán đủ cho nhá</t>
         </is>
       </c>
       <c r="H156" s="3" t="n"/>
@@ -8610,9 +8610,9 @@
       <c r="G157" s="3" t="inlineStr">
         <is>
           <t>1. nó ra ngoài rồi
-2. có quen sao em
+2. có có quen có việc gì không
 3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. ừ anh thanh toán đủ cho nhá</t>
+4. ừ để anh thanh toán cho bên em nhé</t>
         </is>
       </c>
       <c r="H157" s="3" t="n"/>
@@ -8662,10 +8662,10 @@
       </c>
       <c r="G158" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. anh biết bạn ấy có gì không
-3. anh thanh toán một ít trước nhé
-4. ừ anh thanh toán đủ cho nhá</t>
+          <t>1. anh nghe hộ thôi
+2. có quen sao em
+3. giờ trả được một ít trước thôi em
+4. được để anh trả tiền</t>
         </is>
       </c>
       <c r="H158" s="3" t="n"/>
@@ -8714,9 +8714,9 @@
         <is>
           <t>1. tôi là anh nó
 2. có quen sao em
-3. giờ trả được một ít trước thôi em
-4. lúc khác rồi nói
-5. anh đang bận</t>
+3. anh thanh toán một ít trước nhé
+4. anh đang bận
+5. không nói chuyện được</t>
         </is>
       </c>
       <c r="H159" s="3" t="n"/>
@@ -8768,9 +8768,9 @@
       </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ tôi có biết
-3. thanh toán một phần trước nhé em
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
+3. anh thanh toán một ít trước nhé
 4. _silence_
 5. _silence_</t>
         </is>
@@ -8823,8 +8823,8 @@
       </c>
       <c r="G161" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ tôi có biết
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ người quen
 3. anh thanh toán một ít trước nhé hơi kẹt em ạ
 4. _silence_
 5. _silence_</t>
@@ -8879,9 +8879,9 @@
       </c>
       <c r="G162" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. có quen sao em
-3. trả trước một phần có được không em
+          <t>1. tôi là anh nó
+2. ừ ừ người quen
+3. thanh toán một phần trước nhé em
 4. _silence_
 5. _silence_</t>
         </is>
@@ -8935,9 +8935,9 @@
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. có quen sao em
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ tôi có biết
+3. anh thanh toán một ít trước nhé
 4. anh thanh toán một ít trước nhé hơi kẹt em ạ
 5. trả trước một phần có được không em</t>
         </is>
@@ -8991,10 +8991,10 @@
       </c>
       <c r="G164" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. có có quen có việc gì không
-3. anh thanh toán một ít trước nhé
-4. trả trước một phần có được không em
+          <t>1. nó đi chơi rồi
+2. ừ ừ người quen
+3. thanh toán một phần trước nhé em
+4. anh thanh toán cho bên em trước một phần có được không
 5. anh thanh toán một ít trước nhé hơi kẹt em ạ</t>
         </is>
       </c>
@@ -9047,11 +9047,11 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
+          <t>1. nó đi chơi rồi
 2. có có quen có việc gì không
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. anh thanh toán một ít trước nhé
-5. giờ trả được một ít trước thôi em</t>
+3. anh thanh toán một ít trước nhé
+4. giờ trả được một ít trước thôi em
+5. thanh toán một phần trước nhé em</t>
         </is>
       </c>
       <c r="H165" s="3" t="n"/>
@@ -9103,11 +9103,11 @@
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. có có quen có việc gì không
-3. trả trước một phần có được không em
-4. anh trả cho bên em sau không bùng đâu yên tâm
-5. ừ tháng sau trả nhé</t>
+          <t>1. đang nghe hộ không biết đâu
+2. có quen sao em
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. mấy hôm nữa thanh toán nhé
+5. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
         </is>
       </c>
       <c r="H166" s="3" t="n"/>
@@ -9160,9 +9160,9 @@
         <is>
           <t>1. nó ra ngoài rồi
 2. có quen sao em
-3. anh thanh toán một ít trước nhé
-4. ừ biết rồi anh sẽ trả cho bọn em sau
-5. mấy hôm nữa thanh toán nhé</t>
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. anh trả cho bên em sau không bùng đâu yên tâm
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
       <c r="H167" s="3" t="n"/>
@@ -9215,10 +9215,10 @@
       <c r="G168" s="3" t="inlineStr">
         <is>
           <t>1. đang nghe hộ không biết đâu
-2. có có quen có việc gì không
-3. anh thanh toán một ít trước nhé
-4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
-5. anh trả cho bên em sau không bùng đâu yên tâm</t>
+2. ừ ừ người quen
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. anh trả cho bên em sau không bùng đâu yên tâm
+5. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
         </is>
       </c>
       <c r="H168" s="3" t="n"/>
@@ -9270,11 +9270,11 @@
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
+          <t>1. nó ra ngoài rồi
 2. ừ ừ người quen
-3. trả trước một phần có được không em
-4. chẳng nghe thấy gì
-5. nói lại giúm mình với nãy không nghe thấy</t>
+3. giờ trả được một ít trước thôi em
+4. tín hiệu kém quá không nghe thấy gì
+5. nói bé quá nói lại đi em</t>
         </is>
       </c>
       <c r="H169" s="3" t="n"/>
@@ -9325,11 +9325,11 @@
       </c>
       <c r="G170" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ người quen
-3. trả trước một phần có được không em
-4. chẳng nghe thấy gì
-5. không nghe thấy gì hết trơn á</t>
+          <t>1. nó đi chơi rồi
+2. ừ tôi có biết
+3. anh thanh toán một ít trước nhé
+4. nói bé quá nói lại đi em
+5. nghe không rõ nói lại đi em</t>
         </is>
       </c>
       <c r="H170" s="3" t="n"/>
@@ -9381,11 +9381,11 @@
       </c>
       <c r="G171" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ người quen
+          <t>1. đang nghe hộ không biết đâu
+2. anh biết bạn ấy có gì không
 3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. nghe không rõ nói lại đi em
-5. không nghe thấy gì hết trơn á</t>
+4. tín hiệu kém quá không nghe thấy gì
+5. nghe không rõ nói lại đi em</t>
         </is>
       </c>
       <c r="H171" s="3" t="n"/>
@@ -9430,10 +9430,10 @@
       </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
+          <t>1. anh nghe hộ thôi
 2. có có quen có việc gì không
-3. ừ anh thanh toán đủ cho nhá
-4. trả hết rôi mà</t>
+3. ừ để anh thanh toán cho bên em nhé
+4. trả rồi</t>
         </is>
       </c>
       <c r="H172" s="3" t="n"/>
@@ -9495,8 +9495,8 @@
       </c>
       <c r="G174" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ok em nói đi
+          <t>1. đang nghe hộ không biết đâu
+2. nói đi
 3. ủa đã trả rồi mà em</t>
         </is>
       </c>
@@ -9545,8 +9545,8 @@
       </c>
       <c r="G175" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. rồi nói nghe coi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. phải rồi
 3. anh trả được nhiêu còn nợ nhiêu em</t>
         </is>
       </c>
@@ -9595,8 +9595,8 @@
       <c r="G176" s="3" t="inlineStr">
         <is>
           <t>1. đang nghe hộ không biết đâu
-2. nói đi
-3. anh trả được nhiêu còn nợ nhiêu em</t>
+2. ok
+3. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H176" s="3" t="n"/>
@@ -9644,9 +9644,9 @@
       </c>
       <c r="G177" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. được rồi đang nghe đây
-3. mới ung thư mất rồi</t>
+          <t>1. nó đi vắng rồi chưa về
+2. rồi nói nghe coi
+3. chết rồi</t>
         </is>
       </c>
       <c r="H177" s="3" t="n"/>
@@ -9693,9 +9693,9 @@
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ok em nói đi
-3. ừ mất rôi em thông cảm</t>
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
+3. mới ốm mất rồi em ạ</t>
         </is>
       </c>
       <c r="H178" s="3" t="n"/>
@@ -9738,9 +9738,9 @@
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. tôi là anh nó
 2. ok em nói đi
-3. anh đóng nhầm hợp đồng</t>
+3. trả lộn hợp đồng rồi</t>
         </is>
       </c>
       <c r="H179" s="3" t="n"/>
@@ -9788,8 +9788,8 @@
       </c>
       <c r="G180" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. được
+          <t>1. bố cháu đang nghe
+2. ok em nói đi
 3. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
@@ -9838,9 +9838,9 @@
       </c>
       <c r="G181" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. nói nghe xem nào
-3. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
+          <t>1. anh nghe hộ thôi
+2. nói đi
+3. mới ốm mất rồi em ạ</t>
         </is>
       </c>
       <c r="H181" s="3" t="n"/>
@@ -9885,9 +9885,9 @@
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. nói nghe xem nào
-3. lúc khác rồi nói
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. được rồi đang nghe đây
+3. lát rồi gọi lại
 4. đang có việc</t>
         </is>
       </c>
@@ -9938,8 +9938,8 @@
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. được
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. nói nghe xem nào
 3. _silence_
 4. _silence_</t>
         </is>
@@ -9990,8 +9990,8 @@
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ok em nói đi
+          <t>1. nó ra ngoài rồi
+2. ok
 3. _silence_
 4. _silence_</t>
         </is>
@@ -10043,8 +10043,8 @@
       </c>
       <c r="G185" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
+          <t>1. anh nghe hộ thôi
+2. nói nghe xem nào
 3. _silence_
 4. _silence_</t>
         </is>
@@ -10096,10 +10096,10 @@
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok em nói đi
-3. alo alo nghe không có rõ
-4. tín hiệu kém quá không nghe thấy gì</t>
+          <t>1. đang nghe hộ không biết đâu
+2. phải rồi
+3. chẳng nghe thấy gì
+4. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H186" s="3" t="n"/>
@@ -10148,10 +10148,10 @@
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ rồi
+          <t>1. tôi là anh nó
+2. ok em nói đi
 3. chẳng nghe thấy gì
-4. nói bé quá nói lại đi em</t>
+4. nói lại được không em</t>
         </is>
       </c>
       <c r="H187" s="3" t="n"/>
@@ -10201,10 +10201,10 @@
       </c>
       <c r="G188" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. được
+          <t>1. nó ra ngoài rồi
+2. rồi nói nghe coi
 3. nói lại giúm mình với nãy không nghe thấy
-4. tín hiệu kém quá không nghe thấy gì</t>
+4. nói lại giúm mình với nãy không nghe thấy</t>
         </is>
       </c>
       <c r="H188" s="3" t="n"/>
@@ -10278,13 +10278,13 @@
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ rồi
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. nói nghe xem nào
 3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. anh trả cho bên em sau không bùng đâu yên tâm
-6. rồi anh hứa sẽ trả cho bọn em
-7. ủa đã trả rồi mà em</t>
+4. rồi anh hứa sẽ trả cho bọn em
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. chắc chắn sẽ trả cho bên em
+7. tất toán hết rồi em</t>
         </is>
       </c>
       <c r="H190" s="3" t="n"/>
@@ -10331,11 +10331,11 @@
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ
-3. anh đứng tên giùm thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. thanh toán rồi mà em ơi</t>
+          <t>1. đang nghe hộ không biết đâu
+2. được rồi đang nghe đây
+3. anh vay hộ thôi
+4. chắc chắn sẽ trả cho bên em
+5. ủa đã trả rồi mà em</t>
         </is>
       </c>
       <c r="H191" s="3" t="n"/>
@@ -10387,11 +10387,11 @@
       </c>
       <c r="G192" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok em nói đi
-3. anh đứng tên giùm thôi
+          <t>1. nó đi chơi rồi
+2. ừ ừ rồi
+3. anh vay hộ thôi
 4. chắc chắn sẽ trả cho bên em
-5. anh trả được nhiêu còn nợ nhiêu em</t>
+5. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H192" s="3" t="n"/>
@@ -10442,10 +10442,10 @@
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. được
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
+4. hứa sẽ trả yên tâm
 5. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
@@ -10498,11 +10498,11 @@
       </c>
       <c r="G194" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok em nói đi
-3. anh vay hộ thôi
-4. hứa sẽ trả yên tâm
-5. mới ung thư mất rồi</t>
+          <t>1. bố cháu đang nghe
+2. ừ
+3. anh đứng tên giùm thôi
+4. rồi anh hứa sẽ trả cho bọn em
+5. mới ốm mất trong viện tuần trước em ạ</t>
         </is>
       </c>
       <c r="H194" s="3" t="n"/>
@@ -10553,11 +10553,11 @@
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. rồi nói nghe coi
-3. anh vay hộ thôi
-4. hứa sẽ trả yên tâm
-5. ừ mất rôi em thông cảm</t>
+          <t>1. đang nghe hộ không biết đâu
+2. được rồi đang nghe đây
+3. anh đứng tên giùm thôi
+4. chắc chắn sẽ trả cho bên em
+5. chết rồi</t>
         </is>
       </c>
       <c r="H195" s="3" t="n"/>
@@ -10609,10 +10609,10 @@
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. được rồi đang nghe đây
+          <t>1. đang nghe hộ không biết đâu
+2. ừ ừ rồi
 3. anh vay hộ thôi
-4. hứa sẽ trả yên tâm
+4. chắc chắn sẽ trả cho bên em
 5. thanh toán một phần trước nhé em</t>
         </is>
       </c>
@@ -10664,11 +10664,11 @@
       </c>
       <c r="G197" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. nói đi
+          <t>1. đang nghe hộ không biết đâu
+2. rồi nói nghe coi
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. anh thanh toán cho bên em trước một phần có được không</t>
+4. chắc chắn sẽ trả cho bên em
+5. giờ trả được một ít trước thôi em</t>
         </is>
       </c>
       <c r="H197" s="3" t="n"/>
@@ -10715,9 +10715,9 @@
       </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok
-3. anh đứng tên giùm thôi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. được rồi đang nghe đây
+3. anh vay hộ thôi
 4. chắc chắn sẽ trả cho bên em
 5. anh đóng nhầm hợp đồng</t>
         </is>
@@ -10770,11 +10770,11 @@
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ rồi
-3. anh vay hộ thôi
+          <t>1. tôi là anh nó
+2. được rồi đang nghe đây
+3. anh đứng tên giùm thôi
 4. rồi anh hứa sẽ trả cho bọn em
-5. hứa sẽ trả yên tâm</t>
+5. chắc chắn sẽ trả cho bên em</t>
         </is>
       </c>
       <c r="H199" s="3" t="n"/>
@@ -10828,10 +10828,10 @@
       <c r="G200" s="3" t="inlineStr">
         <is>
           <t>1. bố cháu đang nghe
-2. ok em nói đi
-3. anh vay hộ thôi
+2. ừ ừ rồi
+3. anh đứng tên giùm thôi
 4. rồi anh hứa sẽ trả cho bọn em
-5. chắc chắn sẽ trả cho bên em</t>
+5. rồi anh hứa sẽ trả cho bọn em</t>
         </is>
       </c>
       <c r="H200" s="3" t="n"/>
@@ -10883,11 +10883,11 @@
       </c>
       <c r="G201" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. phải rồi
-3. anh đứng tên giùm thôi
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
+3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
-5. hứa sẽ trả yên tâm</t>
+5. chắc chắn sẽ trả cho bên em</t>
         </is>
       </c>
       <c r="H201" s="3" t="n"/>
@@ -10939,8 +10939,8 @@
       </c>
       <c r="G202" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok em nói đi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. nói nghe xem nào
 3. anh đứng tên giùm thôi
 4. hứa sẽ trả yên tâm
 5. anh còn nợ bao tiền đã trả được nhiều chưa</t>
@@ -10995,11 +10995,11 @@
       </c>
       <c r="G203" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. nói nghe xem nào
-3. anh đứng tên giùm thôi
-4. chắc chắn sẽ trả cho bên em
-5. tại nạn chết rồi em</t>
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
+3. anh vay hộ thôi
+4. rồi anh hứa sẽ trả cho bọn em
+5. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
         </is>
       </c>
       <c r="H203" s="3" t="n"/>
@@ -11051,11 +11051,11 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. nó đi chơi rồi
 2. ok em nói đi
-3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. anh thanh toán một ít trước nhé hơi kẹt em ạ</t>
+3. anh đứng tên giùm thôi
+4. hứa sẽ trả yên tâm
+5. anh thanh toán một ít trước nhé</t>
         </is>
       </c>
       <c r="H204" s="3" t="n"/>
@@ -11104,12 +11104,12 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ rồi
-3. anh vay hộ thôi
+          <t>1. nó đi chơi rồi
+2. phải rồi
+3. anh đứng tên giùm thôi
 4. hứa sẽ trả yên tâm
-5. bận rồi
-6. đang đi làm</t>
+5. lúc khác rồi nói
+6. đi học rồi</t>
         </is>
       </c>
       <c r="H205" s="3" t="n"/>
@@ -11163,9 +11163,9 @@
       </c>
       <c r="G206" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ ừ rồi
-3. anh đứng tên giùm thôi
+          <t>1. anh nghe hộ thôi
+2. rồi nói nghe coi
+3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
 5. _silence_
 6. _silence_</t>
@@ -11221,10 +11221,10 @@
       </c>
       <c r="G207" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ok
-3. anh đứng tên giùm thôi
-4. chắc chắn sẽ trả cho bên em
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ừ
+3. anh vay hộ thôi
+4. rồi anh hứa sẽ trả cho bọn em
 5. _silence_
 6. _silence_</t>
         </is>
@@ -11280,8 +11280,8 @@
       </c>
       <c r="G208" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ ừ rồi
+          <t>1. bố cháu đang nghe
+2. nói nghe xem nào
 3. anh vay hộ thôi
 4. chắc chắn sẽ trả cho bên em
 5. _silence_
@@ -11339,12 +11339,12 @@
       </c>
       <c r="G209" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ok
+          <t>1. nó ra ngoài rồi
+2. được rồi đang nghe đây
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
+4. chắc chắn sẽ trả cho bên em
 5. nói bé quá nói lại đi em
-6. nghe không rõ nói lại đi em</t>
+6. alo alo nghe không có rõ</t>
         </is>
       </c>
       <c r="H209" s="3" t="n"/>
@@ -11397,12 +11397,12 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ok
-3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. không nghe thấy gì hết trơn á
-6. nói lại được không em</t>
+          <t>1. đang nghe hộ không biết đâu
+2. ok em nói đi
+3. anh vay hộ thôi
+4. chắc chắn sẽ trả cho bên em
+5. chẳng nghe thấy gì
+6. nói lại giúm mình với nãy không nghe thấy</t>
         </is>
       </c>
       <c r="H210" s="3" t="n"/>
@@ -11456,12 +11456,12 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. nói nghe xem nào
-3. anh đứng tên giùm thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. chẳng nghe thấy gì
-6. tín hiệu kém quá không nghe thấy gì</t>
+          <t>1. bố cháu đang nghe
+2. nói đi
+3. anh vay hộ thôi
+4. chắc chắn sẽ trả cho bên em
+5. nói lại giúm mình với nãy không nghe thấy
+6. chẳng nghe thấy gì</t>
         </is>
       </c>
       <c r="H211" s="3" t="n"/>
@@ -11516,13 +11516,13 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ ừ rồi
-3. khoản nào em anh biết gì đâu
-4. hứa sẽ trả yên tâm
-5. ừ tháng sau trả nhé
+          <t>1. nó đi chơi rồi
+2. ok em nói đi
+3. khoản vay gì anh biết đâu
+4. chắc chắn sẽ trả cho bên em
+5. mấy hôm nữa thanh toán nhé
 6. rồi anh hứa sẽ trả cho bọn em
-7. thanh toán rồi mà em ơi</t>
+7. thanh toán xong hết rồi nhá</t>
         </is>
       </c>
       <c r="H212" s="3" t="n"/>
@@ -11579,13 +11579,13 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. được
+          <t>1. nó đi chơi rồi
+2. ừ ừ rồi
 3. rồi anh hứa sẽ trả cho bọn em
-4. anh thanh toán một ít trước nhé
-5. hứa sẽ trả yên tâm
-6. anh trả cho bên em sau không bùng đâu yên tâm
-7. hứa sẽ trả yên tâm
+4. giờ trả được một ít trước thôi em
+5. rồi anh hứa sẽ trả cho bọn em
+6. ừ anh sẽ tất toán hết cho bên em sau nhé
+7. chắc chắn sẽ trả cho bên em
 8. mới thanh toán đủ cho em rối</t>
         </is>
       </c>
@@ -11641,13 +11641,13 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. hứa sẽ trả yên tâm
-5. ừ biết rồi anh sẽ trả cho bọn em sau
+          <t>1. anh nghe hộ thôi
+2. ok
+3. giờ trả được một ít trước thôi em
+4. rồi anh hứa sẽ trả cho bọn em
+5. anh trả cho bên em sau không bùng đâu yên tâm
 6. hứa sẽ trả yên tâm
-7. thanh toán xong hết rồi nhá</t>
+7. thanh toán rồi mà em ơi</t>
         </is>
       </c>
       <c r="H214" s="3" t="n"/>
@@ -11702,12 +11702,12 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. nói đi
-3. bùng không thanh toán
-4. chắc chắn sẽ trả cho bên em
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
+3. đang khó khăn tôi không trả
+4. hứa sẽ trả yên tâm
 5. anh trả cho bên em sau không bùng đâu yên tâm
-6. chắc chắn sẽ trả cho bên em
+6. rồi anh hứa sẽ trả cho bọn em
 7. thanh toán xong hết rồi nhá</t>
         </is>
       </c>
@@ -11766,10 +11766,10 @@
           <t>1. nó ra ngoài rồi
 2. ông xã đang nghe ạ
 3. anh đứng tên giùm thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+4. chắc chắn sẽ trả cho bên em
+5. ừ anh sẽ tất toán hết cho bên em sau nhé
 6. chắc chắn sẽ trả cho bên em
-7. trả hết rôi mà</t>
+7. ủa đã trả rồi mà em</t>
         </is>
       </c>
       <c r="H216" s="3" t="n"/>
@@ -11822,12 +11822,12 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>1. được rồi đang nghe đây
-2. anh vay hộ thôi
+          <t>1. được
+2. anh đứng tên giùm thôi
 3. rồi anh hứa sẽ trả cho bọn em
-4. ừ biết rồi anh sẽ trả cho bọn em sau
-5. rồi anh hứa sẽ trả cho bọn em
-6. mới thanh toán đủ cho em rối</t>
+4. anh trả cho bên em sau không bùng đâu yên tâm
+5. chắc chắn sẽ trả cho bên em
+6. thanh toán xong hết rồi nhá</t>
         </is>
       </c>
       <c r="H217" s="3" t="n"/>
@@ -11880,12 +11880,12 @@
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
-          <t>1. ông xã đang nghe ạ
-2. anh đứng tên giùm thôi
+          <t>1. chồng đang nghe sao thế
+2. anh vay hộ thôi
 3. chắc chắn sẽ trả cho bên em
-4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
-5. hứa sẽ trả yên tâm
-6. trả rồi</t>
+4. ừ tháng sau trả nhé
+5. chắc chắn sẽ trả cho bên em
+6. mới thanh toán đủ cho em rối</t>
         </is>
       </c>
       <c r="H218" s="3" t="n"/>
@@ -11949,9 +11949,9 @@
       </c>
       <c r="G220" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok em nói đi
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. nói đi
+3. anh thanh toán một ít trước nhé
 4. trả hết rôi mà</t>
         </is>
       </c>
@@ -12002,10 +12002,10 @@
       </c>
       <c r="G221" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ok em nói đi
-3. anh thanh toán một ít trước nhé
-4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. phải rồi
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. anh trả được nhiêu còn nợ nhiêu em</t>
         </is>
       </c>
       <c r="H221" s="3" t="n"/>
@@ -12055,10 +12055,10 @@
       </c>
       <c r="G222" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ok
 3. trả trước một phần có được không em
-4. anh không biết khoản vay nào</t>
+4. không biết khoản vay nào luôn</t>
         </is>
       </c>
       <c r="H222" s="3" t="n"/>
@@ -12108,10 +12108,10 @@
       </c>
       <c r="G223" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok em nói đi
-3. anh thanh toán cho bên em trước một phần có được không
-4. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
+          <t>1. bố cháu đang nghe
+2. nói đi
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. ốm chết rồi</t>
         </is>
       </c>
       <c r="H223" s="3" t="n"/>
@@ -12161,10 +12161,10 @@
       </c>
       <c r="G224" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. được rồi đang nghe đây
-3. anh thanh toán một ít trước nhé
-4. anh thanh toán một ít trước nhé hơi kẹt em ạ</t>
+          <t>1. tôi là anh nó
+2. nói đi
+3. trả trước một phần có được không em
+4. trả trước một phần có được không em</t>
         </is>
       </c>
       <c r="H224" s="3" t="n"/>
@@ -12214,10 +12214,10 @@
       </c>
       <c r="G225" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. được
-3. anh thanh toán một ít trước nhé
-4. thanh toán cái gì không trả tiền đâu</t>
+          <t>1. anh nghe hộ thôi
+2. ừ
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. tôi không trả đấy</t>
         </is>
       </c>
       <c r="H225" s="3" t="n"/>
@@ -12266,10 +12266,10 @@
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. được rồi đang nghe đây
-3. giờ trả được một ít trước thôi em
-4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. phải rồi
+3. anh thanh toán cho bên em trước một phần có được không
+4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H226" s="3" t="n"/>
@@ -12318,9 +12318,9 @@
       </c>
       <c r="G227" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
 2. nói đi
-3. anh thanh toán một ít trước nhé
+3. anh thanh toán cho bên em trước một phần có được không
 4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
@@ -12370,8 +12370,8 @@
       </c>
       <c r="G228" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. nói nghe xem nào
+          <t>1. bố cháu đang nghe
+2. phải rồi
 3. anh thanh toán một ít trước nhé hơi kẹt em ạ
 4. giờ trả được một ít trước thôi em</t>
         </is>
@@ -12422,10 +12422,10 @@
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok
-3. trả trước một phần có được không em
-4. đang khó khăn tôi không trả</t>
+          <t>1. bố cháu đang nghe
+2. được
+3. anh thanh toán cho bên em trước một phần có được không
+4. dạo này kẹt anh không trả được</t>
         </is>
       </c>
       <c r="H229" s="3" t="n"/>
@@ -12475,10 +12475,10 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. được rồi đang nghe đây
-3. trả trước một phần có được không em
-4. mấy hôm nữa thanh toán nhé</t>
+          <t>1. tôi là anh nó
+2. ok
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. ừ tháng sau trả nhé</t>
         </is>
       </c>
       <c r="H230" s="3" t="n"/>
@@ -12528,9 +12528,9 @@
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. nói nghe xem nào
-3. trả trước một phần có được không em
+          <t>1. bố cháu đang nghe
+2. ừ ừ rồi
+3. thanh toán một phần trước nhé em
 4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
@@ -12580,10 +12580,10 @@
       </c>
       <c r="G232" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. được rồi đang nghe đây
-3. thanh toán một phần trước nhé em
-4. mới ốm mất trong viện tuần trước em ạ</t>
+          <t>1. anh nghe hộ thôi
+2. nói nghe xem nào
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. ốm chết rồi</t>
         </is>
       </c>
       <c r="H232" s="3" t="n"/>
@@ -12633,10 +12633,10 @@
       </c>
       <c r="G233" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. phải rồi
-3. anh thanh toán một ít trước nhé
-4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. được rồi đang nghe đây
+3. trả trước một phần có được không em
+4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H233" s="3" t="n"/>
@@ -12686,10 +12686,10 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. rồi nói nghe coi
-3. anh thanh toán một ít trước nhé
-4. anh không biết khoản vay nào</t>
+          <t>1. bố cháu đang nghe
+2. nói nghe xem nào
+3. thanh toán một phần trước nhé em
+4. khoản vay gì anh biết đâu</t>
         </is>
       </c>
       <c r="H234" s="3" t="n"/>
@@ -12740,9 +12740,9 @@
       <c r="G235" s="3" t="inlineStr">
         <is>
           <t>1. nó đi vắng rồi chưa về
-2. ok
-3. anh thanh toán một ít trước nhé
-4. mất rồi em</t>
+2. ừ ừ rồi
+3. anh thanh toán cho bên em trước một phần có được không
+4. tại nạn chết rồi em</t>
         </is>
       </c>
       <c r="H235" s="3" t="n"/>
@@ -12792,10 +12792,10 @@
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok
-3. anh thanh toán cho bên em trước một phần có được không
-4. anh thanh toán một ít trước nhé</t>
+          <t>1. anh nghe hộ thôi
+2. nói nghe xem nào
+3. anh thanh toán một ít trước nhé hơi kẹt em ạ
+4. trả trước một phần có được không em</t>
         </is>
       </c>
       <c r="H236" s="3" t="n"/>
@@ -12845,10 +12845,10 @@
       </c>
       <c r="G237" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ
+          <t>1. nó đi chơi rồi
+2. nói đi
 3. giờ trả được một ít trước thôi em
-4. không trả không có tiền</t>
+4. hết tiền rồi không trả được</t>
         </is>
       </c>
       <c r="H237" s="3" t="n"/>
@@ -12898,10 +12898,10 @@
       </c>
       <c r="G238" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. phải rồi
-3. anh thanh toán một ít trước nhé hơi kẹt em ạ
-4. ừ biết rồi anh sẽ trả cho bọn em sau</t>
+          <t>1. anh nghe hộ thôi
+2. được rồi đang nghe đây
+3. trả trước một phần có được không em
+4. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
         </is>
       </c>
       <c r="H238" s="3" t="n"/>
@@ -12948,11 +12948,11 @@
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. rồi nói nghe coi
-3. giờ trả được một ít trước thôi em
-4. không nói chuyện được
-5. đang có việc</t>
+          <t>1. nó ra ngoài rồi
+2. được rồi đang nghe đây
+3. thanh toán một phần trước nhé em
+4. lúc khác rồi nói
+5. đang đi làm</t>
         </is>
       </c>
       <c r="H239" s="3" t="n"/>
@@ -13004,9 +13004,9 @@
       </c>
       <c r="G240" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. nói đi
-3. thanh toán một phần trước nhé em
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
+3. giờ trả được một ít trước thôi em
 4. _silence_
 5. _silence_</t>
         </is>
@@ -13059,9 +13059,9 @@
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. tôi là anh nó
 2. rồi nói nghe coi
-3. anh thanh toán cho bên em trước một phần có được không
+3. giờ trả được một ít trước thôi em
 4. _silence_
 5. _silence_</t>
         </is>
@@ -13115,8 +13115,8 @@
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. nói nghe xem nào
+          <t>1. nó đi chơi rồi
+2. được
 3. anh thanh toán cho bên em trước một phần có được không
 4. _silence_
 5. _silence_</t>
@@ -13171,11 +13171,11 @@
       </c>
       <c r="G243" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. được
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. nói nghe xem nào
 3. trả trước một phần có được không em
-4. nói lại được không em
-5. chẳng nghe thấy gì</t>
+4. alo alo nghe không có rõ
+5. alo alo nghe không có rõ</t>
         </is>
       </c>
       <c r="H243" s="3" t="n"/>
@@ -13226,10 +13226,10 @@
       </c>
       <c r="G244" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ok em nói đi
-3. anh thanh toán một ít trước nhé
-4. tín hiệu kém quá không nghe thấy gì
+          <t>1. nó đi vắng rồi chưa về
+2. ừ
+3. giờ trả được một ít trước thôi em
+4. nói bé quá nói lại đi em
 5. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
@@ -13283,10 +13283,10 @@
       <c r="G245" s="3" t="inlineStr">
         <is>
           <t>1. tôi là anh nó
-2. nói đi
+2. ừ ừ rồi
 3. giờ trả được một ít trước thôi em
-4. tín hiệu kém quá không nghe thấy gì
-5. nói lại giúm mình với nãy không nghe thấy</t>
+4. nói lại giúm mình với nãy không nghe thấy
+5. alo alo nghe không có rõ</t>
         </is>
       </c>
       <c r="H245" s="3" t="n"/>
@@ -13358,12 +13358,12 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ rồi
-3. anh đứng tên giùm thôi
+          <t>1. nó ra ngoài rồi
+2. ok em nói đi
+3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
-5. ừ tháng sau trả nhé
-6. trả hết rôi mà</t>
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. mới thanh toán đủ cho em rối</t>
         </is>
       </c>
       <c r="H247" s="3" t="n"/>
@@ -13417,12 +13417,12 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. rồi nói nghe coi
-3. anh đứng tên giùm thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. ừ biết rồi anh sẽ trả cho bọn em sau
-6. anh trả được nhiêu còn nợ nhiêu em</t>
+          <t>1. nó đi chơi rồi
+2. nói nghe xem nào
+3. anh vay hộ thôi
+4. chắc chắn sẽ trả cho bên em
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H248" s="3" t="n"/>
@@ -13476,11 +13476,11 @@
       </c>
       <c r="G249" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ok em nói đi
-3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. được rồi đang nghe đây
+3. anh đứng tên giùm thôi
+4. chắc chắn sẽ trả cho bên em
+5. anh trả cho bên em sau không bùng đâu yên tâm
 6. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
@@ -13536,11 +13536,11 @@
       <c r="G250" s="3" t="inlineStr">
         <is>
           <t>1. tôi là anh nó
-2. được rồi đang nghe đây
-3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. anh trả cho bên em sau không bùng đâu yên tâm
-6. đột quỵ chết rồi em ạ</t>
+2. rồi nói nghe coi
+3. anh vay hộ thôi
+4. chắc chắn sẽ trả cho bên em
+5. ừ anh sẽ tất toán hết cho bên em sau nhé
+6. ốm chết rồi</t>
         </is>
       </c>
       <c r="H250" s="3" t="n"/>
@@ -13594,12 +13594,12 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. rồi nói nghe coi
+          <t>1. nó ra ngoài rồi
+2. được
 3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
-5. ừ tháng sau trả nhé
-6. thanh toán một phần trước nhé em</t>
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. giờ trả được một ít trước thôi em</t>
         </is>
       </c>
       <c r="H251" s="3" t="n"/>
@@ -13653,12 +13653,12 @@
       </c>
       <c r="G252" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ rồi
+          <t>1. nó ra ngoài rồi
+2. nói nghe xem nào
 3. anh vay hộ thôi
-4. hứa sẽ trả yên tâm
-5. mấy hôm nữa thanh toán nhé
-6. dạo này kẹt anh không trả được</t>
+4. chắc chắn sẽ trả cho bên em
+5. anh trả cho bên em sau không bùng đâu yên tâm
+6. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H252" s="3" t="n"/>
@@ -13712,12 +13712,12 @@
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. nó ra ngoài rồi
 2. nói đi
 3. anh vay hộ thôi
 4. rồi anh hứa sẽ trả cho bọn em
-5. ừ tháng sau trả nhé
-6. anh trả được nhiêu còn nợ nhiêu em</t>
+5. ừ biết rồi anh sẽ trả cho bọn em sau
+6. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H253" s="3" t="n"/>
@@ -13771,12 +13771,12 @@
       </c>
       <c r="G254" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. được rồi đang nghe đây
-3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. ừ anh sẽ tất toán hết cho bên em sau nhé
-6. anh không biết khoản vay nào</t>
+          <t>1. nó đi vắng rồi chưa về
+2. được
+3. anh vay hộ thôi
+4. rồi anh hứa sẽ trả cho bọn em
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. không biết khoản vay nào luôn</t>
         </is>
       </c>
       <c r="H254" s="3" t="n"/>
@@ -13830,12 +13830,12 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. nói nghe xem nào
+          <t>1. bố cháu đang nghe
+2. phải rồi
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
+4. hứa sẽ trả yên tâm
 5. anh trả cho bên em sau không bùng đâu yên tâm
-6. anh thanh toán một ít trước nhé</t>
+6. anh thanh toán cho bên em trước một phần có được không</t>
         </is>
       </c>
       <c r="H255" s="3" t="n"/>
@@ -13889,12 +13889,12 @@
       </c>
       <c r="G256" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. rồi nói nghe coi
-3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. ừ anh sẽ tất toán hết cho bên em sau nhé
-6. dạo này kẹt anh không trả được</t>
+          <t>1. bố cháu đang nghe
+2. nói đi
+3. anh đứng tên giùm thôi
+4. chắc chắn sẽ trả cho bên em
+5. anh trả cho bên em sau không bùng đâu yên tâm
+6. tôi không trả đấy</t>
         </is>
       </c>
       <c r="H256" s="3" t="n"/>
@@ -13948,8 +13948,8 @@
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ok em nói đi
 3. anh đứng tên giùm thôi
 4. rồi anh hứa sẽ trả cho bọn em
 5. ừ anh sẽ tất toán hết cho bên em sau nhé
@@ -14007,12 +14007,12 @@
       </c>
       <c r="G258" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ok
+          <t>1. bố cháu đang nghe
+2. rồi nói nghe coi
 3. anh vay hộ thôi
-4. hứa sẽ trả yên tâm
-5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
-6. anh trả cho bên em sau không bùng đâu yên tâm</t>
+4. chắc chắn sẽ trả cho bên em
+5. mấy hôm nữa thanh toán nhé
+6. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
       <c r="H258" s="3" t="n"/>
@@ -14066,12 +14066,12 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. nói đi
+          <t>1. nó đi chơi rồi
+2. phải rồi
 3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. anh trả cho bên em sau không bùng đâu yên tâm
-6. mới ung thư mất rồi</t>
+4. rồi anh hứa sẽ trả cho bọn em
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. ốm chết rồi</t>
         </is>
       </c>
       <c r="H259" s="3" t="n"/>
@@ -14125,12 +14125,12 @@
       </c>
       <c r="G260" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
-3. anh đứng tên giùm thôi
+          <t>1. bố cháu đang nghe
+2. ừ
+3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
-5. ừ biết rồi anh sẽ trả cho bọn em sau
-6. anh còn nợ bao tiền đã trả được nhiều chưa</t>
+5. ừ anh sẽ tất toán hết cho bên em sau nhé
+6. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H260" s="3" t="n"/>
@@ -14184,12 +14184,12 @@
       </c>
       <c r="G261" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. nói nghe xem nào
+          <t>1. nó đi chơi rồi
+2. ok
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. ừ tháng sau trả nhé
-6. khoản nào em anh biết gì đâu</t>
+4. chắc chắn sẽ trả cho bên em
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. anh không biết khoản vay nào</t>
         </is>
       </c>
       <c r="H261" s="3" t="n"/>
@@ -14243,12 +14243,12 @@
       </c>
       <c r="G262" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ừ
-3. anh vay hộ thôi
+          <t>1. tôi là anh nó
+2. rồi nói nghe coi
+3. anh đứng tên giùm thôi
 4. hứa sẽ trả yên tâm
-5. anh trả cho bên em sau không bùng đâu yên tâm
-6. mới ốm mất rồi em ạ</t>
+5. ừ anh sẽ tất toán hết cho bên em sau nhé
+6. mới ốm mất trong viện tuần trước em ạ</t>
         </is>
       </c>
       <c r="H262" s="3" t="n"/>
@@ -14303,11 +14303,11 @@
       <c r="G263" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. ừ
-3. anh đứng tên giùm thôi
-4. chắc chắn sẽ trả cho bên em
-5. mấy hôm nữa thanh toán nhé
-6. anh thanh toán một ít trước nhé</t>
+2. ok
+3. anh vay hộ thôi
+4. hứa sẽ trả yên tâm
+5. ừ tháng sau trả nhé
+6. trả trước một phần có được không em</t>
         </is>
       </c>
       <c r="H263" s="3" t="n"/>
@@ -14361,12 +14361,12 @@
       </c>
       <c r="G264" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. nói nghe xem nào
-3. anh đứng tên giùm thôi
-4. chắc chắn sẽ trả cho bên em
-5. ừ anh sẽ tất toán hết cho bên em sau nhé
-6. không trả không có tiền</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ
+3. anh vay hộ thôi
+4. hứa sẽ trả yên tâm
+5. anh trả cho bên em sau không bùng đâu yên tâm
+6. không trả đâu</t>
         </is>
       </c>
       <c r="H264" s="3" t="n"/>
@@ -14421,11 +14421,11 @@
       <c r="G265" s="3" t="inlineStr">
         <is>
           <t>1. đang nghe hộ không biết đâu
-2. phải rồi
+2. ừ
 3. anh vay hộ thôi
 4. chắc chắn sẽ trả cho bên em
-5. anh trả cho bên em sau không bùng đâu yên tâm
-6. mấy hôm nữa thanh toán nhé</t>
+5. ừ anh sẽ tất toán hết cho bên em sau nhé
+6. ừ tháng sau trả nhé</t>
         </is>
       </c>
       <c r="H265" s="3" t="n"/>
@@ -14481,12 +14481,12 @@
       <c r="G266" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. nói đi
+2. nói nghe xem nào
 3. anh vay hộ thôi
 4. hứa sẽ trả yên tâm
-5. ừ biết rồi anh sẽ trả cho bọn em sau
-6. lát rồi gọi lại
-7. anh đang đi trên đường</t>
+5. ừ tháng sau trả nhé
+6. lúc khác rồi nói
+7. đi học rồi</t>
         </is>
       </c>
       <c r="H266" s="3" t="n"/>
@@ -14542,11 +14542,11 @@
       </c>
       <c r="G267" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. rồi nói nghe coi
+          <t>1. bố cháu đang nghe
+2. nói đi
 3. anh vay hộ thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. ừ anh sẽ tất toán hết cho bên em sau nhé
+4. hứa sẽ trả yên tâm
+5. ừ tháng sau trả nhé
 6. _silence_
 7. _silence_</t>
         </is>
@@ -14604,11 +14604,11 @@
       </c>
       <c r="G268" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
+          <t>1. đang nghe hộ không biết đâu
+2. nói đi
 3. anh đứng tên giùm thôi
 4. rồi anh hứa sẽ trả cho bọn em
-5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+5. ừ biết rồi anh sẽ trả cho bọn em sau
 6. _silence_
 7. _silence_</t>
         </is>
@@ -14667,9 +14667,9 @@
       <c r="G269" s="3" t="inlineStr">
         <is>
           <t>1. bố cháu đang nghe
-2. ok
-3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
+2. nói nghe xem nào
+3. anh vay hộ thôi
+4. rồi anh hứa sẽ trả cho bọn em
 5. anh trả cho bên em sau không bùng đâu yên tâm
 6. _silence_
 7. _silence_</t>
@@ -14728,13 +14728,13 @@
       </c>
       <c r="G270" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ok em nói đi
+          <t>1. bố cháu đang nghe
+2. phải rồi
 3. anh đứng tên giùm thôi
-4. rồi anh hứa sẽ trả cho bọn em
-5. ừ tháng sau trả nhé
+4. chắc chắn sẽ trả cho bên em
+5. anh trả cho bên em sau không bùng đâu yên tâm
 6. chẳng nghe thấy gì
-7. tín hiệu kém quá không nghe thấy gì</t>
+7. alo alo nghe không có rõ</t>
         </is>
       </c>
       <c r="H270" s="3" t="n"/>
@@ -14790,13 +14790,13 @@
       </c>
       <c r="G271" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ
-3. anh vay hộ thôi
+          <t>1. nó ra ngoài rồi
+2. ok
+3. anh đứng tên giùm thôi
 4. rồi anh hứa sẽ trả cho bọn em
-5. ừ biết rồi anh sẽ trả cho bọn em sau
-6. nói lại được không em
-7. nói lại được không em</t>
+5. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+6. không nghe thấy gì hết trơn á
+7. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H271" s="3" t="n"/>
@@ -14852,13 +14852,13 @@
       </c>
       <c r="G272" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. nói đi
+          <t>1. bố cháu đang nghe
+2. phải rồi
 3. anh đứng tên giùm thôi
-4. hứa sẽ trả yên tâm
-5. ừ biết rồi anh sẽ trả cho bọn em sau
-6. không nghe thấy gì hết trơn á
-7. nói bé quá nói lại đi em</t>
+4. chắc chắn sẽ trả cho bên em
+5. ừ tháng sau trả nhé
+6. chẳng nghe thấy gì
+7. tín hiệu kém quá không nghe thấy gì</t>
         </is>
       </c>
       <c r="H272" s="3" t="n"/>
@@ -14911,12 +14911,12 @@
       </c>
       <c r="G273" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. phải rồi
-3. được rồi anh sẽ thanh toán cho em sau nhé phải mấy
+          <t>1. nó đi vắng rồi chưa về
+2. rồi nói nghe coi
+3. mấy hôm nữa thanh toán nhé
 4. rồi anh hứa sẽ trả cho bọn em
-5. ừ anh sẽ tất toán hết cho bên em sau nhé
-6. mới thanh toán đủ cho em rối</t>
+5. ừ biết rồi anh sẽ trả cho bọn em sau
+6. trả rồi</t>
         </is>
       </c>
       <c r="H273" s="3" t="n"/>
@@ -14980,10 +14980,10 @@
       </c>
       <c r="G275" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. nói đi
-3. tôi không trả đấy
-4. thanh toán xong hết rồi nhá</t>
+          <t>1. nó đi chơi rồi
+2. nói nghe xem nào
+3. không trả đâu
+4. trả rồi</t>
         </is>
       </c>
       <c r="H275" s="3" t="n"/>
@@ -15033,10 +15033,10 @@
       </c>
       <c r="G276" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. rồi nói nghe coi
-3. bùng không thanh toán
-4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
+          <t>1. nó đi chơi rồi
+2. phải rồi
+3. đang khó khăn tôi không trả
+4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H276" s="3" t="n"/>
@@ -15086,9 +15086,9 @@
       </c>
       <c r="G277" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. phải rồi
-3. tôi không trả đấy
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ok
+3. đang khó khăn tôi không trả
 4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
@@ -15139,10 +15139,10 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. nó đi vắng rồi chưa về
 2. ok
 3. tôi không trả đấy
-4. mất rồi em</t>
+4. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
         </is>
       </c>
       <c r="H278" s="3" t="n"/>
@@ -15192,10 +15192,10 @@
       </c>
       <c r="G279" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. được
-3. không trả không có tiền
-4. ừ tháng sau trả nhé</t>
+          <t>1. nó đi vắng rồi chưa về
+2. ok
+3. hết tiền rồi không trả được
+4. mấy hôm nữa thanh toán nhé</t>
         </is>
       </c>
       <c r="H279" s="3" t="n"/>
@@ -15245,10 +15245,10 @@
       </c>
       <c r="G280" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ok
-3. thanh toán cái gì không trả tiền đâu
-4. bùng không thanh toán</t>
+          <t>1. anh nghe hộ thôi
+2. rồi nói nghe coi
+3. đang khó khăn tôi không trả
+4. dạo này kẹt anh không trả được</t>
         </is>
       </c>
       <c r="H280" s="3" t="n"/>
@@ -15297,9 +15297,9 @@
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. được rồi đang nghe đây
-3. dạo này kẹt anh không trả được
+          <t>1. nó đi vắng rồi chưa về
+2. ok em nói đi
+3. thanh toán cái gì không trả tiền đâu
 4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
@@ -15349,10 +15349,10 @@
       </c>
       <c r="G282" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ ừ rồi
-3. đang khó khăn tôi không trả
-4. anh không biết khoản vay nào</t>
+          <t>1. anh nghe hộ thôi
+2. nói đi
+3. không trả đâu
+4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
       <c r="H282" s="3" t="n"/>
@@ -15401,9 +15401,9 @@
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. anh nghe hộ thôi
 2. nói đi
-3. bùng không thanh toán
+3. không trả không có tiền
 4. anh trả cho bên em sau không bùng đâu yên tâm</t>
         </is>
       </c>
@@ -15453,10 +15453,10 @@
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. nó đi chơi rồi
 2. được
 3. bùng không thanh toán
-4. dạo này kẹt anh không trả được</t>
+4. tôi không trả đấy</t>
         </is>
       </c>
       <c r="H284" s="3" t="n"/>
@@ -15506,10 +15506,10 @@
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok em nói đi
-3. hết tiền rồi không trả được
-4. anh thanh toán cho bên em trước một phần có được không</t>
+          <t>1. tôi là anh nó
+2. nói đi
+3. tôi không trả đấy
+4. trả trước một phần có được không em</t>
         </is>
       </c>
       <c r="H285" s="3" t="n"/>
@@ -15559,10 +15559,10 @@
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. được rồi đang nghe đây
-3. không trả đâu
-4. anh thanh toán một ít trước nhé hơi kẹt em ạ</t>
+          <t>1. bố cháu đang nghe
+2. rồi nói nghe coi
+3. không trả không có tiền
+4. giờ trả được một ít trước thôi em</t>
         </is>
       </c>
       <c r="H286" s="3" t="n"/>
@@ -15611,10 +15611,10 @@
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. được rồi đang nghe đây
-3. thanh toán cái gì không trả tiền đâu
-4. tại nạn chết rồi em</t>
+          <t>1. đang nghe hộ không biết đâu
+2. nói đi
+3. không trả không có tiền
+4. mất rồi em</t>
         </is>
       </c>
       <c r="H287" s="3" t="n"/>
@@ -15665,9 +15665,9 @@
       <c r="G288" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. ok em nói đi
-3. đang khó khăn tôi không trả
-4. anh trả được nhiêu còn nợ nhiêu em</t>
+2. ok
+3. không trả đâu
+4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H288" s="3" t="n"/>
@@ -15717,9 +15717,9 @@
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. được
-3. không trả không có tiền
+          <t>1. bố cháu đang nghe
+2. ok
+3. dạo này kẹt anh không trả được
 4. không biết khoản vay nào luôn</t>
         </is>
       </c>
@@ -15770,9 +15770,9 @@
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. ok
-3. tôi không trả đấy
+          <t>1. bố cháu đang nghe
+2. ừ ừ rồi
+3. dạo này kẹt anh không trả được
 4. mới bị tai nạn chết hôm qua đau sót quá em ạ</t>
         </is>
       </c>
@@ -15823,10 +15823,10 @@
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ
-3. tôi không trả đấy
-4. ừ biết rồi anh sẽ trả cho bọn em sau</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. được rồi đang nghe đây
+3. không trả đâu
+4. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
         </is>
       </c>
       <c r="H291" s="3" t="n"/>
@@ -15876,10 +15876,10 @@
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. được rồi đang nghe đây
-3. hết tiền rồi không trả được
-4. không trả đâu</t>
+          <t>1. nó đi vắng rồi chưa về
+2. nói đi
+3. thanh toán cái gì không trả tiền đâu
+4. thanh toán cái gì không trả tiền đâu</t>
         </is>
       </c>
       <c r="H292" s="3" t="n"/>
@@ -15929,10 +15929,10 @@
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ok em nói đi
-3. hết tiền rồi không trả được
-4. trả trước một phần có được không em</t>
+          <t>1. tôi là anh nó
+2. nói đi
+3. đang khó khăn tôi không trả
+4. thanh toán một phần trước nhé em</t>
         </is>
       </c>
       <c r="H293" s="3" t="n"/>
@@ -15979,11 +15979,11 @@
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. ừ ừ rồi
-3. tôi không trả đấy
-4. lúc khác rồi nói
-5. đang đi làm</t>
+          <t>1. nó đi chơi rồi
+2. nói nghe xem nào
+3. không trả đâu
+4. chưa tiện để nói chuyện
+5. lát rồi gọi lại</t>
         </is>
       </c>
       <c r="H294" s="3" t="n"/>
@@ -16035,9 +16035,9 @@
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ
-3. bùng không thanh toán
+          <t>1. nó đi vắng rồi chưa về
+2. ok
+3. không trả không có tiền
 4. _silence_
 5. _silence_</t>
         </is>
@@ -16091,8 +16091,8 @@
       <c r="G296" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. nói nghe xem nào
-3. bùng không thanh toán
+2. rồi nói nghe coi
+3. dạo này kẹt anh không trả được
 4. _silence_
 5. _silence_</t>
         </is>
@@ -16147,8 +16147,8 @@
       <c r="G297" s="3" t="inlineStr">
         <is>
           <t>1. nó đi chơi rồi
-2. ừ ừ rồi
-3. tôi không trả đấy
+2. được rồi đang nghe đây
+3. không trả không có tiền
 4. _silence_
 5. _silence_</t>
         </is>
@@ -16202,11 +16202,11 @@
       </c>
       <c r="G298" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. rồi nói nghe coi
-3. thanh toán cái gì không trả tiền đâu
-4. không nghe thấy gì hết trơn á
-5. nói lại giúm mình với nãy không nghe thấy</t>
+          <t>1. bố cháu đang nghe
+2. ok em nói đi
+3. đang khó khăn tôi không trả
+4. tín hiệu kém quá không nghe thấy gì
+5. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H298" s="3" t="n"/>
@@ -16257,11 +16257,11 @@
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. nó đi chơi rồi
 2. ok
-3. tôi không trả đấy
-4. nói bé quá nói lại đi em
-5. nghe không rõ nói lại đi em</t>
+3. không trả đâu
+4. không nghe thấy gì hết trơn á
+5. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H299" s="3" t="n"/>
@@ -16313,11 +16313,11 @@
       </c>
       <c r="G300" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. nói đi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. được
 3. đang khó khăn tôi không trả
 4. nói lại giúm mình với nãy không nghe thấy
-5. nói lại được không em</t>
+5. nói bé quá nói lại đi em</t>
         </is>
       </c>
       <c r="H300" s="3" t="n"/>
@@ -16381,10 +16381,10 @@
       </c>
       <c r="G302" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. nói nghe xem nào
-3. anh vay hộ thôi
-4. mới thanh toán đủ cho em rối</t>
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. rồi nói nghe coi
+3. anh đứng tên giùm thôi
+4. thanh toán xong hết rồi nhá</t>
         </is>
       </c>
       <c r="H302" s="3" t="n"/>
@@ -16434,10 +16434,10 @@
       </c>
       <c r="G303" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. đang nghe hộ không biết đâu
 2. ừ
-3. anh đứng tên giùm thôi
-4. anh trả được nhiêu còn nợ nhiêu em</t>
+3. anh vay hộ thôi
+4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H303" s="3" t="n"/>
@@ -16487,10 +16487,10 @@
       </c>
       <c r="G304" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ rồi
+          <t>1. nó đi vắng rồi chưa về
+2. được rồi đang nghe đây
 3. anh đứng tên giùm thôi
-4. khoản vay gì anh biết đâu</t>
+4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
       <c r="H304" s="3" t="n"/>
@@ -16540,10 +16540,10 @@
       </c>
       <c r="G305" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. nó ra ngoài rồi
 2. ok
-3. anh đứng tên giùm thôi
-4. tại nạn chết rồi em</t>
+3. anh vay hộ thôi
+4. mới ung thư mất rồi</t>
         </is>
       </c>
       <c r="H305" s="3" t="n"/>
@@ -16593,10 +16593,10 @@
       </c>
       <c r="G306" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ừ ừ rồi
-3. anh vay hộ thôi
-4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
+          <t>1. đang nghe hộ không biết đâu
+2. nói đi
+3. anh đứng tên giùm thôi
+4. ừ tháng sau trả nhé</t>
         </is>
       </c>
       <c r="H306" s="3" t="n"/>
@@ -16646,10 +16646,10 @@
       </c>
       <c r="G307" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. phải rồi
-3. anh vay hộ thôi
-4. tôi không trả đấy</t>
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. ok
+3. anh đứng tên giùm thôi
+4. thanh toán cái gì không trả tiền đâu</t>
         </is>
       </c>
       <c r="H307" s="3" t="n"/>
@@ -16698,10 +16698,10 @@
       </c>
       <c r="G308" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ rồi
-3. anh vay hộ thôi
-4. anh trả được nhiêu còn nợ nhiêu em</t>
+          <t>1. bố cháu đang nghe
+2. rồi nói nghe coi
+3. anh đứng tên giùm thôi
+4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
         </is>
       </c>
       <c r="H308" s="3" t="n"/>
@@ -16750,10 +16750,10 @@
       </c>
       <c r="G309" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ok em nói đi
+          <t>1. anh nghe hộ thôi
+2. phải rồi
 3. anh vay hộ thôi
-4. khoản vay gì anh biết đâu</t>
+4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
       <c r="H309" s="3" t="n"/>
@@ -16802,10 +16802,10 @@
       </c>
       <c r="G310" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. phải rồi
+          <t>1. anh nghe hộ thôi
+2. nói đi
 3. anh vay hộ thôi
-4. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
+4. mấy hôm nữa thanh toán nhé</t>
         </is>
       </c>
       <c r="H310" s="3" t="n"/>
@@ -16854,10 +16854,10 @@
       </c>
       <c r="G311" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. phải rồi
-3. anh đứng tên giùm thôi
-4. tôi không trả đấy</t>
+          <t>1. nó đi chơi rồi
+2. nói nghe xem nào
+3. anh vay hộ thôi
+4. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H311" s="3" t="n"/>
@@ -16907,10 +16907,10 @@
       </c>
       <c r="G312" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. được
-3. anh đứng tên giùm thôi
-4. anh thanh toán một ít trước nhé</t>
+          <t>1. nó đi vắng rồi chưa về
+2. ừ ừ rồi
+3. anh vay hộ thôi
+4. anh thanh toán cho bên em trước một phần có được không</t>
         </is>
       </c>
       <c r="H312" s="3" t="n"/>
@@ -16960,10 +16960,10 @@
       </c>
       <c r="G313" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ừ
-3. anh vay hộ thôi
-4. thanh toán một phần trước nhé em</t>
+          <t>1. anh nghe hộ thôi
+2. được rồi đang nghe đây
+3. anh đứng tên giùm thôi
+4. giờ trả được một ít trước thôi em</t>
         </is>
       </c>
       <c r="H313" s="3" t="n"/>
@@ -17012,10 +17012,10 @@
       </c>
       <c r="G314" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ ừ rồi
+          <t>1. tôi là anh nó
+2. ok em nói đi
 3. anh đứng tên giùm thôi
-4. tại nạn chết rồi em</t>
+4. chết rồi</t>
         </is>
       </c>
       <c r="H314" s="3" t="n"/>
@@ -17065,9 +17065,9 @@
       </c>
       <c r="G315" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+          <t>1. anh nghe hộ thôi
 2. được
-3. anh vay hộ thôi
+3. anh đứng tên giùm thôi
 4. anh trả được nhiêu còn nợ nhiêu em</t>
         </is>
       </c>
@@ -17118,10 +17118,10 @@
       </c>
       <c r="G316" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. phải rồi
+          <t>1. bố cháu đang nghe
+2. ừ
 3. anh đứng tên giùm thôi
-4. không biết khoản vay nào luôn</t>
+4. khoản nào em anh biết gì đâu</t>
         </is>
       </c>
       <c r="H316" s="3" t="n"/>
@@ -17171,10 +17171,10 @@
       </c>
       <c r="G317" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ
+          <t>1. bố cháu đang nghe
+2. ok em nói đi
 3. anh đứng tên giùm thôi
-4. mới ốm mất trong viện tuần trước em ạ</t>
+4. mới ốm mất rồi em ạ</t>
         </is>
       </c>
       <c r="H317" s="3" t="n"/>
@@ -17224,7 +17224,7 @@
       </c>
       <c r="G318" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
 2. được
 3. anh vay hộ thôi
 4. anh trả cho bên em sau không bùng đâu yên tâm</t>
@@ -17277,10 +17277,10 @@
       </c>
       <c r="G319" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. anh nghe hộ thôi
 2. ok em nói đi
-3. anh đứng tên giùm thôi
-4. hết tiền rồi không trả được</t>
+3. anh vay hộ thôi
+4. không trả đâu</t>
         </is>
       </c>
       <c r="H319" s="3" t="n"/>
@@ -17330,10 +17330,10 @@
       </c>
       <c r="G320" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
+          <t>1. anh nghe hộ thôi
 2. ok em nói đi
-3. anh đứng tên giùm thôi
-4. giờ trả được một ít trước thôi em</t>
+3. anh vay hộ thôi
+4. anh thanh toán cho bên em trước một phần có được không</t>
         </is>
       </c>
       <c r="H320" s="3" t="n"/>
@@ -17381,10 +17381,10 @@
       <c r="G321" s="3" t="inlineStr">
         <is>
           <t>1. tôi là anh nó
-2. được
+2. ok em nói đi
 3. anh vay hộ thôi
-4. đang đi làm
-5. đang có việc</t>
+4. bận rồi
+5. không nói chuyện được</t>
         </is>
       </c>
       <c r="H321" s="3" t="n"/>
@@ -17436,8 +17436,8 @@
       </c>
       <c r="G322" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ
+          <t>1. nó đi chơi rồi
+2. rồi nói nghe coi
 3. anh vay hộ thôi
 4. _silence_
 5. _silence_</t>
@@ -17491,7 +17491,7 @@
       </c>
       <c r="G323" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. tôi là anh nó
 2. nói đi
 3. anh vay hộ thôi
 4. _silence_
@@ -17547,8 +17547,8 @@
       </c>
       <c r="G324" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ừ
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. được
 3. anh vay hộ thôi
 4. _silence_
 5. _silence_</t>
@@ -17603,11 +17603,11 @@
       </c>
       <c r="G325" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ok
-3. anh đứng tên giùm thôi
-4. chẳng nghe thấy gì
-5. nói lại giúm mình với nãy không nghe thấy</t>
+          <t>1. đang nghe hộ không biết đâu
+2. phải rồi
+3. anh vay hộ thôi
+4. nghe không rõ nói lại đi em
+5. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
       <c r="H325" s="3" t="n"/>
@@ -17658,11 +17658,11 @@
       </c>
       <c r="G326" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. được rồi đang nghe đây
+          <t>1. nó đi vắng rồi chưa về
+2. phải rồi
 3. anh đứng tên giùm thôi
-4. nghe không rõ nói lại đi em
-5. tín hiệu kém quá không nghe thấy gì</t>
+4. nói lại được không em
+5. nói bé quá nói lại đi em</t>
         </is>
       </c>
       <c r="H326" s="3" t="n"/>
@@ -17714,11 +17714,11 @@
       </c>
       <c r="G327" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. rồi nói nghe coi
-3. anh vay hộ thôi
-4. chẳng nghe thấy gì
-5. alo alo nghe không có rõ</t>
+          <t>1. tôi là anh nó
+2. ừ
+3. anh đứng tên giùm thôi
+4. alo alo nghe không có rõ
+5. nói lại được không em</t>
         </is>
       </c>
       <c r="H327" s="3" t="n"/>
@@ -17782,9 +17782,9 @@
       </c>
       <c r="G329" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
+          <t>1. bố cháu đang nghe
 2. phải rồi
-3. anh không biết khoản vay nào
+3. khoản nào em anh biết gì đâu
 4. tất toán hết rồi em</t>
         </is>
       </c>
@@ -17835,10 +17835,10 @@
       </c>
       <c r="G330" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ
+          <t>1. tôi là anh nó
+2. ok em nói đi
 3. khoản nào em anh biết gì đâu
-4. anh còn nợ nhiều không trả được bao nhiêu rồi</t>
+4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H330" s="3" t="n"/>
@@ -17888,10 +17888,10 @@
       </c>
       <c r="G331" s="3" t="inlineStr">
         <is>
-          <t>1. đang nghe hộ không biết đâu
-2. ừ ừ rồi
-3. anh không biết khoản vay nào
-4. khoản nào em anh biết gì đâu</t>
+          <t>1. nó đi chơi rồi
+2. ok em nói đi
+3. khoản nào em anh biết gì đâu
+4. khoản vay gì anh biết đâu</t>
         </is>
       </c>
       <c r="H331" s="3" t="n"/>
@@ -17941,10 +17941,10 @@
       </c>
       <c r="G332" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. ok
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. được rồi đang nghe đây
 3. anh không biết khoản vay nào
-4. tại nạn chết rồi em</t>
+4. mất rồi em</t>
         </is>
       </c>
       <c r="H332" s="3" t="n"/>
@@ -17994,10 +17994,10 @@
       </c>
       <c r="G333" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. được rồi đang nghe đây
-3. khoản vay gì anh biết đâu
-4. ừ biết rồi anh sẽ trả cho bọn em sau</t>
+          <t>1. tôi là anh nó
+2. ừ
+3. anh không biết khoản vay nào
+4. ừ anh sẽ tất toán hết cho bên em sau nhé</t>
         </is>
       </c>
       <c r="H333" s="3" t="n"/>
@@ -18047,10 +18047,10 @@
       </c>
       <c r="G334" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
+          <t>1. anh nghe hộ thôi
 2. được rồi đang nghe đây
-3. anh không biết khoản vay nào
-4. đang khó khăn tôi không trả</t>
+3. không biết khoản vay nào luôn
+4. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H334" s="3" t="n"/>
@@ -18099,7 +18099,7 @@
       </c>
       <c r="G335" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
+          <t>1. nó đi vắng rồi chưa về
 2. ừ
 3. anh không biết khoản vay nào
 4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
@@ -18151,10 +18151,10 @@
       </c>
       <c r="G336" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. được
-3. không biết khoản vay nào luôn
-4. không biết khoản vay nào luôn</t>
+          <t>1. nó đi vắng rồi chưa về
+2. ok
+3. khoản nào em anh biết gì đâu
+4. anh không biết khoản vay nào</t>
         </is>
       </c>
       <c r="H336" s="3" t="n"/>
@@ -18203,10 +18203,10 @@
       </c>
       <c r="G337" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. được rồi đang nghe đây
-3. khoản vay gì anh biết đâu
-4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
+          <t>1. tôi là anh nó
+2. ừ
+3. khoản nào em anh biết gì đâu
+4. ừ biết rồi anh sẽ trả cho bọn em sau</t>
         </is>
       </c>
       <c r="H337" s="3" t="n"/>
@@ -18255,10 +18255,10 @@
       </c>
       <c r="G338" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. được
-3. anh không biết khoản vay nào
-4. tôi không trả đấy</t>
+          <t>1. bố cháu đang nghe
+2. ok
+3. khoản vay gì anh biết đâu
+4. bùng không thanh toán</t>
         </is>
       </c>
       <c r="H338" s="3" t="n"/>
@@ -18308,8 +18308,8 @@
       </c>
       <c r="G339" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. được
+          <t>1. nó ra ngoài rồi
+2. được rồi đang nghe đây
 3. khoản nào em anh biết gì đâu
 4. anh thanh toán một ít trước nhé</t>
         </is>
@@ -18361,10 +18361,10 @@
       </c>
       <c r="G340" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. được
-3. khoản nào em anh biết gì đâu
-4. thanh toán một phần trước nhé em</t>
+          <t>1. nó đi vắng rồi chưa về
+2. rồi nói nghe coi
+3. anh không biết khoản vay nào
+4. anh thanh toán một ít trước nhé</t>
         </is>
       </c>
       <c r="H340" s="3" t="n"/>
@@ -18413,10 +18413,10 @@
       </c>
       <c r="G341" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi vắng rồi chưa về
-2. nói đi
-3. khoản nào em anh biết gì đâu
-4. ừ mất rôi em thông cảm</t>
+          <t>1. bố cháu đang nghe
+2. phải rồi
+3. khoản vay gì anh biết đâu
+4. mới ung thư mất rồi</t>
         </is>
       </c>
       <c r="H341" s="3" t="n"/>
@@ -18466,10 +18466,10 @@
       </c>
       <c r="G342" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
+          <t>1. anh nghe hộ thôi
 2. được
-3. không biết khoản vay nào luôn
-4. anh trả được nhiêu còn nợ nhiêu em</t>
+3. khoản vay gì anh biết đâu
+4. anh còn nợ bao tiền đã trả được nhiều chưa</t>
         </is>
       </c>
       <c r="H342" s="3" t="n"/>
@@ -18519,10 +18519,10 @@
       </c>
       <c r="G343" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. nói nghe xem nào
-3. không biết khoản vay nào luôn
-4. khoản nào em anh biết gì đâu</t>
+          <t>1. nó đi chơi rồi
+2. ừ
+3. khoản nào em anh biết gì đâu
+4. không biết khoản vay nào luôn</t>
         </is>
       </c>
       <c r="H343" s="3" t="n"/>
@@ -18572,10 +18572,10 @@
       </c>
       <c r="G344" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. nói đi
-3. không biết khoản vay nào luôn
-4. chết rồi</t>
+          <t>1. nó đi vắng rồi chưa về
+2. phải rồi
+3. anh không biết khoản vay nào
+4. mới ốm mất rồi em ạ</t>
         </is>
       </c>
       <c r="H344" s="3" t="n"/>
@@ -18625,9 +18625,9 @@
       </c>
       <c r="G345" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. rồi nói nghe coi
-3. anh không biết khoản vay nào
+          <t>1. nó ra ngoài rồi
+2. nói đi
+3. không biết khoản vay nào luôn
 4. được rồi anh sẽ thanh toán cho em sau nhé phải mấy</t>
         </is>
       </c>
@@ -18678,10 +18678,10 @@
       </c>
       <c r="G346" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. ok
+          <t>1. bố cháu đang nghe
+2. nói đi
 3. khoản nào em anh biết gì đâu
-4. không trả đâu</t>
+4. dạo này kẹt anh không trả được</t>
         </is>
       </c>
       <c r="H346" s="3" t="n"/>
@@ -18731,9 +18731,9 @@
       </c>
       <c r="G347" s="3" t="inlineStr">
         <is>
-          <t>1. nó ra ngoài rồi
-2. ừ
-3. không biết khoản vay nào luôn
+          <t>1. anh nghe hộ thôi
+2. được rồi đang nghe đây
+3. khoản vay gì anh biết đâu
 4. thanh toán một phần trước nhé em</t>
         </is>
       </c>
@@ -18781,11 +18781,11 @@
       </c>
       <c r="G348" s="3" t="inlineStr">
         <is>
-          <t>1. tôi là anh nó
-2. ừ ừ rồi
+          <t>1. bố cháu đang nghe
+2. nói đi
 3. khoản vay gì anh biết đâu
-4. lát rồi gọi lại
-5. lát rồi gọi lại</t>
+4. anh đang bận
+5. lúc khác rồi nói</t>
         </is>
       </c>
       <c r="H348" s="3" t="n"/>
@@ -18837,9 +18837,9 @@
       </c>
       <c r="G349" s="3" t="inlineStr">
         <is>
-          <t>1. bố cháu đang nghe
-2. phải rồi
-3. anh không biết khoản vay nào
+          <t>1. đang nghe hộ không biết đâu
+2. ừ
+3. khoản nào em anh biết gì đâu
 4. _silence_
 5. _silence_</t>
         </is>
@@ -18892,8 +18892,8 @@
       </c>
       <c r="G350" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. ừ ừ rồi
+          <t>1. tôi là anh nó
+2. nói nghe xem nào
 3. khoản vay gì anh biết đâu
 4. _silence_
 5. _silence_</t>
@@ -18948,9 +18948,9 @@
       </c>
       <c r="G351" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi chơi rồi
-2. ok
-3. khoản vay gì anh biết đâu
+          <t>1. nó ra ngoài rồi
+2. nói đi
+3. không biết khoản vay nào luôn
 4. _silence_
 5. _silence_</t>
         </is>
@@ -19004,11 +19004,11 @@
       </c>
       <c r="G352" s="3" t="inlineStr">
         <is>
-          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
-2. rồi nói nghe coi
+          <t>1. nó đi ra ngoài rồi không có nhà đâu
+2. phải rồi
 3. anh không biết khoản vay nào
-4. nói lại giúm mình với nãy không nghe thấy
-5. nói lại được không em</t>
+4. tín hiệu kém quá không nghe thấy gì
+5. alo alo nghe không có rõ</t>
         </is>
       </c>
       <c r="H352" s="3" t="n"/>
@@ -19059,10 +19059,10 @@
       </c>
       <c r="G353" s="3" t="inlineStr">
         <is>
-          <t>1. nó đi ra ngoài rồi không có nhà đâu
-2. nói nghe xem nào
-3. không biết khoản vay nào luôn
-4. nói lại giúm mình với nãy không nghe thấy
+          <t>1. nó đi vắng rồi chưa về
+2. ừ
+3. anh không biết khoản vay nào
+4. alo alo nghe không có rõ
 5. không nghe thấy gì hết trơn á</t>
         </is>
       </c>
@@ -19115,10 +19115,10 @@
       </c>
       <c r="G354" s="3" t="inlineStr">
         <is>
-          <t>1. anh nghe hộ thôi
-2. phải rồi
-3. anh không biết khoản vay nào
-4. không nghe thấy gì hết trơn á
+          <t>1. tí anh nhắn lại cho nó nó ra ngoài rồi
+2. ừ
+3. khoản nào em anh biết gì đâu
+4. nghe không rõ nói lại đi em
 5. nghe không rõ nói lại đi em</t>
         </is>
       </c>

</xml_diff>